<commit_message>
feat(engine): implement and stabilize 2-pool FOMP model
This commit introduces a new, fully functional two-pool First-Order
Mineralization Process (FOMP) model and includes several related fixes
and repository improvements.

- Implements a mathematically precise decay model using the analytical
  solution `decay = stock * (1 - exp(-k))`.
- Refactors the FOMP calculation into a pure function and a wrapper to
  ensure compatibility with the ODYM solver, resolving conflicts with
  the final mass balance stock accounting.
- Corrects stock calculation to use a beginning-of-period convention,
  ensuring plots correctly display an initial stock of zero.
- Fixes related bugs in the Monte Carlo simulation and plotting functions
  that arose during development.
- Adds `kaleido` dependency to `requirements.txt` for robust image export.

chore: Performs a repository cleanup by removing the `Archive` directory,
clearing output folders, and adding a `.gitignore` file.
</commit_message>
<xml_diff>
--- a/biodym_mfa_tool/data/02_output/results_scientific.xlsx
+++ b/biodym_mfa_tool/data/02_output/results_scientific.xlsx
@@ -6408,13 +6408,13 @@
         <v>2025</v>
       </c>
       <c r="C288">
-        <v>57953.8933825696</v>
+        <v>57953.89338256961</v>
       </c>
       <c r="D288">
-        <v>13817.34511860948</v>
+        <v>13817.34511860949</v>
       </c>
       <c r="E288">
-        <v>44136.54826396011</v>
+        <v>44136.54826396013</v>
       </c>
       <c r="F288">
         <v>0</v>
@@ -6428,13 +6428,13 @@
         <v>2026</v>
       </c>
       <c r="C289">
-        <v>66788.27293134169</v>
+        <v>66788.27293134171</v>
       </c>
       <c r="D289">
         <v>15923.63451539543</v>
       </c>
       <c r="E289">
-        <v>50864.63841594626</v>
+        <v>50864.63841594627</v>
       </c>
       <c r="F289">
         <v>0</v>
@@ -6448,13 +6448,13 @@
         <v>2027</v>
       </c>
       <c r="C290">
-        <v>51237.05740699392</v>
+        <v>51237.05740699393</v>
       </c>
       <c r="D290">
-        <v>12215.9196515237</v>
+        <v>12215.91965152371</v>
       </c>
       <c r="E290">
-        <v>39021.13775547021</v>
+        <v>39021.13775547023</v>
       </c>
       <c r="F290">
         <v>0</v>
@@ -6468,13 +6468,13 @@
         <v>2028</v>
       </c>
       <c r="C291">
-        <v>53264.12821275886</v>
+        <v>53264.12821275887</v>
       </c>
       <c r="D291">
-        <v>12699.21309857856</v>
+        <v>12699.21309857857</v>
       </c>
       <c r="E291">
-        <v>40564.91511418029</v>
+        <v>40564.9151141803</v>
       </c>
       <c r="F291">
         <v>0</v>
@@ -6508,13 +6508,13 @@
         <v>2030</v>
       </c>
       <c r="C293">
-        <v>65121.37004990324</v>
+        <v>65121.37004990325</v>
       </c>
       <c r="D293">
         <v>15526.21216725399</v>
       </c>
       <c r="E293">
-        <v>49595.15788264925</v>
+        <v>49595.15788264926</v>
       </c>
       <c r="F293">
         <v>0</v>
@@ -6528,13 +6528,13 @@
         <v>2031</v>
       </c>
       <c r="C294">
-        <v>78258.51262490547</v>
+        <v>78258.51262490549</v>
       </c>
       <c r="D294">
         <v>18658.36468085506</v>
       </c>
       <c r="E294">
-        <v>59600.14794405041</v>
+        <v>59600.14794405042</v>
       </c>
       <c r="F294">
         <v>0</v>
@@ -6548,13 +6548,13 @@
         <v>2032</v>
       </c>
       <c r="C295">
-        <v>74599.21427713789</v>
+        <v>74599.2142771379</v>
       </c>
       <c r="D295">
         <v>17785.9161668391</v>
       </c>
       <c r="E295">
-        <v>56813.29811029878</v>
+        <v>56813.29811029879</v>
       </c>
       <c r="F295">
         <v>0</v>
@@ -6568,13 +6568,13 @@
         <v>2033</v>
       </c>
       <c r="C296">
-        <v>83229.825223869</v>
+        <v>83229.82522386902</v>
       </c>
       <c r="D296">
         <v>19843.62313137756</v>
       </c>
       <c r="E296">
-        <v>63386.20209249144</v>
+        <v>63386.20209249145</v>
       </c>
       <c r="F296">
         <v>0</v>
@@ -6588,13 +6588,13 @@
         <v>2034</v>
       </c>
       <c r="C297">
-        <v>73723.90626539658</v>
+        <v>73723.9062653966</v>
       </c>
       <c r="D297">
         <v>17577.22556509687</v>
       </c>
       <c r="E297">
-        <v>56146.68070029971</v>
+        <v>56146.68070029972</v>
       </c>
       <c r="F297">
         <v>0</v>
@@ -6608,13 +6608,13 @@
         <v>2035</v>
       </c>
       <c r="C298">
-        <v>70449.43694571852</v>
+        <v>70449.43694571854</v>
       </c>
       <c r="D298">
         <v>16796.52784093158</v>
       </c>
       <c r="E298">
-        <v>53652.90910478694</v>
+        <v>53652.90910478695</v>
       </c>
       <c r="F298">
         <v>0</v>
@@ -6628,13 +6628,13 @@
         <v>2036</v>
       </c>
       <c r="C299">
-        <v>70732.71985272031</v>
+        <v>70732.71985272033</v>
       </c>
       <c r="D299">
-        <v>16864.06804338886</v>
+        <v>16864.06804338887</v>
       </c>
       <c r="E299">
-        <v>53868.65180933145</v>
+        <v>53868.65180933146</v>
       </c>
       <c r="F299">
         <v>0</v>
@@ -6648,13 +6648,13 @@
         <v>2037</v>
       </c>
       <c r="C300">
-        <v>84821.27627132577</v>
+        <v>84821.27627132578</v>
       </c>
       <c r="D300">
-        <v>20223.05628208795</v>
+        <v>20223.05628208796</v>
       </c>
       <c r="E300">
-        <v>64598.21998923781</v>
+        <v>64598.21998923782</v>
       </c>
       <c r="F300">
         <v>0</v>
@@ -6668,13 +6668,13 @@
         <v>2038</v>
       </c>
       <c r="C301">
-        <v>82418.58191055825</v>
+        <v>82418.58191055826</v>
       </c>
       <c r="D301">
-        <v>19650.2068105588</v>
+        <v>19650.20681055881</v>
       </c>
       <c r="E301">
-        <v>62768.37509999944</v>
+        <v>62768.37509999945</v>
       </c>
       <c r="F301">
         <v>0</v>
@@ -6688,13 +6688,13 @@
         <v>2039</v>
       </c>
       <c r="C302">
-        <v>72483.70931147336</v>
+        <v>72483.70931147337</v>
       </c>
       <c r="D302">
-        <v>17281.53828116782</v>
+        <v>17281.53828116783</v>
       </c>
       <c r="E302">
-        <v>55202.17103030553</v>
+        <v>55202.17103030554</v>
       </c>
       <c r="F302">
         <v>0</v>
@@ -6708,13 +6708,13 @@
         <v>2040</v>
       </c>
       <c r="C303">
-        <v>91229.27089785061</v>
+        <v>91229.27089785063</v>
       </c>
       <c r="D303">
         <v>21750.84791272789</v>
       </c>
       <c r="E303">
-        <v>69478.42298512271</v>
+        <v>69478.42298512273</v>
       </c>
       <c r="F303">
         <v>0</v>
@@ -6728,13 +6728,13 @@
         <v>2041</v>
       </c>
       <c r="C304">
-        <v>75507.45721353272</v>
+        <v>75507.45721353273</v>
       </c>
       <c r="D304">
         <v>18002.45910073422</v>
       </c>
       <c r="E304">
-        <v>57504.99811279849</v>
+        <v>57504.9981127985</v>
       </c>
       <c r="F304">
         <v>0</v>
@@ -6748,13 +6748,13 @@
         <v>2042</v>
       </c>
       <c r="C305">
-        <v>83746.7789177088</v>
+        <v>83746.77891770881</v>
       </c>
       <c r="D305">
-        <v>19966.87503355731</v>
+        <v>19966.87503355732</v>
       </c>
       <c r="E305">
-        <v>63779.90388415148</v>
+        <v>63779.90388415149</v>
       </c>
       <c r="F305">
         <v>0</v>
@@ -6768,13 +6768,13 @@
         <v>2043</v>
       </c>
       <c r="C306">
-        <v>81911.06305458808</v>
+        <v>81911.0630545881</v>
       </c>
       <c r="D306">
         <v>19529.20435881929</v>
       </c>
       <c r="E306">
-        <v>62381.85869576879</v>
+        <v>62381.85869576881</v>
       </c>
       <c r="F306">
         <v>0</v>
@@ -6788,13 +6788,13 @@
         <v>2044</v>
       </c>
       <c r="C307">
-        <v>73807.50452860985</v>
+        <v>73807.50452860986</v>
       </c>
       <c r="D307">
-        <v>17597.15703107291</v>
+        <v>17597.15703107292</v>
       </c>
       <c r="E307">
-        <v>56210.34749753692</v>
+        <v>56210.34749753694</v>
       </c>
       <c r="F307">
         <v>0</v>
@@ -6808,7 +6808,7 @@
         <v>2045</v>
       </c>
       <c r="C308">
-        <v>76743.64214808078</v>
+        <v>76743.64214808079</v>
       </c>
       <c r="D308">
         <v>18297.18984053666</v>
@@ -6828,10 +6828,10 @@
         <v>2046</v>
       </c>
       <c r="C309">
-        <v>85047.46479224972</v>
+        <v>85047.46479224974</v>
       </c>
       <c r="D309">
-        <v>20276.98406282984</v>
+        <v>20276.98406282985</v>
       </c>
       <c r="E309">
         <v>64770.48072941988</v>
@@ -6848,13 +6848,13 @@
         <v>2047</v>
       </c>
       <c r="C310">
-        <v>87463.96212920183</v>
+        <v>87463.96212920184</v>
       </c>
       <c r="D310">
-        <v>20853.1244346674</v>
+        <v>20853.12443466741</v>
       </c>
       <c r="E310">
-        <v>66610.83769453442</v>
+        <v>66610.83769453444</v>
       </c>
       <c r="F310">
         <v>0</v>
@@ -6868,13 +6868,13 @@
         <v>2048</v>
       </c>
       <c r="C311">
-        <v>72264.15433881662</v>
+        <v>72264.15433881663</v>
       </c>
       <c r="D311">
-        <v>17229.19206846941</v>
+        <v>17229.19206846942</v>
       </c>
       <c r="E311">
-        <v>55034.9622703472</v>
+        <v>55034.96227034721</v>
       </c>
       <c r="F311">
         <v>0</v>
@@ -6888,13 +6888,13 @@
         <v>2049</v>
       </c>
       <c r="C312">
-        <v>86124.25555154201</v>
+        <v>86124.25555154202</v>
       </c>
       <c r="D312">
-        <v>20533.71210426538</v>
+        <v>20533.71210426539</v>
       </c>
       <c r="E312">
-        <v>65590.54344727662</v>
+        <v>65590.54344727664</v>
       </c>
       <c r="F312">
         <v>0</v>
@@ -6908,13 +6908,13 @@
         <v>2050</v>
       </c>
       <c r="C313">
-        <v>85455.65718520385</v>
+        <v>85455.65718520386</v>
       </c>
       <c r="D313">
         <v>20374.3051372054</v>
       </c>
       <c r="E313">
-        <v>65081.35204799844</v>
+        <v>65081.35204799845</v>
       </c>
       <c r="F313">
         <v>0</v>
@@ -6948,16 +6948,16 @@
         <v>2026</v>
       </c>
       <c r="C315">
-        <v>0</v>
+        <v>32796.58685675026</v>
       </c>
       <c r="D315">
         <v>0</v>
       </c>
       <c r="E315">
-        <v>0</v>
+        <v>32796.58685675026</v>
       </c>
       <c r="F315">
-        <v>0</v>
+        <v>32796.58685675026</v>
       </c>
     </row>
     <row r="316" spans="1:6">
@@ -6968,16 +6968,16 @@
         <v>2027</v>
       </c>
       <c r="C316">
-        <v>0</v>
+        <v>57383.93074828545</v>
       </c>
       <c r="D316">
         <v>0</v>
       </c>
       <c r="E316">
-        <v>0</v>
+        <v>57383.93074828545</v>
       </c>
       <c r="F316">
-        <v>0</v>
+        <v>57383.93074828545</v>
       </c>
     </row>
     <row r="317" spans="1:6">
@@ -6988,16 +6988,16 @@
         <v>2028</v>
       </c>
       <c r="C317">
-        <v>0</v>
+        <v>63527.20104949955</v>
       </c>
       <c r="D317">
         <v>0</v>
       </c>
       <c r="E317">
-        <v>0</v>
+        <v>63527.20104949955</v>
       </c>
       <c r="F317">
-        <v>0</v>
+        <v>63527.20104949955</v>
       </c>
     </row>
     <row r="318" spans="1:6">
@@ -7008,16 +7008,16 @@
         <v>2029</v>
       </c>
       <c r="C318">
-        <v>0</v>
+        <v>68145.76004186686</v>
       </c>
       <c r="D318">
         <v>0</v>
       </c>
       <c r="E318">
-        <v>0</v>
+        <v>68145.76004186686</v>
       </c>
       <c r="F318">
-        <v>0</v>
+        <v>68145.76004186686</v>
       </c>
     </row>
     <row r="319" spans="1:6">
@@ -7028,16 +7028,16 @@
         <v>2030</v>
       </c>
       <c r="C319">
-        <v>0</v>
+        <v>79742.02009536952</v>
       </c>
       <c r="D319">
         <v>0</v>
       </c>
       <c r="E319">
-        <v>0</v>
+        <v>79742.02009536952</v>
       </c>
       <c r="F319">
-        <v>0</v>
+        <v>79742.02009536952</v>
       </c>
     </row>
     <row r="320" spans="1:6">
@@ -7048,16 +7048,16 @@
         <v>2031</v>
       </c>
       <c r="C320">
-        <v>0</v>
+        <v>83838.94531260688</v>
       </c>
       <c r="D320">
         <v>0</v>
       </c>
       <c r="E320">
-        <v>0</v>
+        <v>83838.94531260688</v>
       </c>
       <c r="F320">
-        <v>0</v>
+        <v>83838.94531260688</v>
       </c>
     </row>
     <row r="321" spans="1:6">
@@ -7068,16 +7068,16 @@
         <v>2032</v>
       </c>
       <c r="C321">
-        <v>0</v>
+        <v>92820.518523587</v>
       </c>
       <c r="D321">
         <v>0</v>
       </c>
       <c r="E321">
-        <v>0</v>
+        <v>92820.518523587</v>
       </c>
       <c r="F321">
-        <v>0</v>
+        <v>92820.518523587</v>
       </c>
     </row>
     <row r="322" spans="1:6">
@@ -7088,16 +7088,16 @@
         <v>2033</v>
       </c>
       <c r="C322">
-        <v>0</v>
+        <v>96131.31108837241</v>
       </c>
       <c r="D322">
         <v>0</v>
       </c>
       <c r="E322">
-        <v>0</v>
+        <v>96131.31108837241</v>
       </c>
       <c r="F322">
-        <v>0</v>
+        <v>96131.31108837241</v>
       </c>
     </row>
     <row r="323" spans="1:6">
@@ -7108,16 +7108,16 @@
         <v>2034</v>
       </c>
       <c r="C323">
-        <v>0</v>
+        <v>102154.5607737415</v>
       </c>
       <c r="D323">
         <v>0</v>
       </c>
       <c r="E323">
-        <v>0</v>
+        <v>102154.5607737415</v>
       </c>
       <c r="F323">
-        <v>0</v>
+        <v>102154.5607737415</v>
       </c>
     </row>
     <row r="324" spans="1:6">
@@ -7128,16 +7128,16 @@
         <v>2035</v>
       </c>
       <c r="C324">
-        <v>0</v>
+        <v>100850.4977098972</v>
       </c>
       <c r="D324">
         <v>0</v>
       </c>
       <c r="E324">
-        <v>0</v>
+        <v>100850.4977098972</v>
       </c>
       <c r="F324">
-        <v>0</v>
+        <v>100850.4977098972</v>
       </c>
     </row>
     <row r="325" spans="1:6">
@@ -7148,16 +7148,16 @@
         <v>2036</v>
       </c>
       <c r="C325">
-        <v>0</v>
+        <v>98204.37046313824</v>
       </c>
       <c r="D325">
         <v>0</v>
       </c>
       <c r="E325">
-        <v>0</v>
+        <v>98204.37046313824</v>
       </c>
       <c r="F325">
-        <v>0</v>
+        <v>98204.37046313824</v>
       </c>
     </row>
     <row r="326" spans="1:6">
@@ -7168,16 +7168,16 @@
         <v>2037</v>
       </c>
       <c r="C326">
-        <v>0</v>
+        <v>96466.05101983748</v>
       </c>
       <c r="D326">
         <v>0</v>
       </c>
       <c r="E326">
-        <v>0</v>
+        <v>96466.05101983748</v>
       </c>
       <c r="F326">
-        <v>0</v>
+        <v>96466.05101983748</v>
       </c>
     </row>
     <row r="327" spans="1:6">
@@ -7188,16 +7188,16 @@
         <v>2038</v>
       </c>
       <c r="C327">
-        <v>0</v>
+        <v>101729.3739547848</v>
       </c>
       <c r="D327">
         <v>0</v>
       </c>
       <c r="E327">
-        <v>0</v>
+        <v>101729.3739547848</v>
       </c>
       <c r="F327">
-        <v>0</v>
+        <v>101729.3739547848</v>
       </c>
     </row>
     <row r="328" spans="1:6">
@@ -7208,16 +7208,16 @@
         <v>2039</v>
       </c>
       <c r="C328">
-        <v>0</v>
+        <v>103510.7240469388</v>
       </c>
       <c r="D328">
         <v>0</v>
       </c>
       <c r="E328">
-        <v>0</v>
+        <v>103510.7240469388</v>
       </c>
       <c r="F328">
-        <v>0</v>
+        <v>103510.7240469388</v>
       </c>
     </row>
     <row r="329" spans="1:6">
@@ -7228,16 +7228,16 @@
         <v>2040</v>
       </c>
       <c r="C329">
-        <v>0</v>
+        <v>99786.3616189317</v>
       </c>
       <c r="D329">
         <v>0</v>
       </c>
       <c r="E329">
-        <v>0</v>
+        <v>99786.3616189317</v>
       </c>
       <c r="F329">
-        <v>0</v>
+        <v>99786.3616189317</v>
       </c>
     </row>
     <row r="330" spans="1:6">
@@ -7248,16 +7248,16 @@
         <v>2041</v>
       </c>
       <c r="C330">
-        <v>0</v>
+        <v>105625.7687010712</v>
       </c>
       <c r="D330">
         <v>0</v>
       </c>
       <c r="E330">
-        <v>0</v>
+        <v>105625.7687010712</v>
       </c>
       <c r="F330">
-        <v>0</v>
+        <v>105625.7687010712</v>
       </c>
     </row>
     <row r="331" spans="1:6">
@@ -7268,16 +7268,16 @@
         <v>2042</v>
       </c>
       <c r="C331">
-        <v>0</v>
+        <v>101929.2012371724</v>
       </c>
       <c r="D331">
         <v>0</v>
       </c>
       <c r="E331">
-        <v>0</v>
+        <v>101929.2012371724</v>
       </c>
       <c r="F331">
-        <v>0</v>
+        <v>101929.2012371724</v>
       </c>
     </row>
     <row r="332" spans="1:6">
@@ -7288,16 +7288,16 @@
         <v>2043</v>
       </c>
       <c r="C332">
-        <v>0</v>
+        <v>102975.0698501281</v>
       </c>
       <c r="D332">
         <v>0</v>
       </c>
       <c r="E332">
-        <v>0</v>
+        <v>102975.0698501281</v>
       </c>
       <c r="F332">
-        <v>0</v>
+        <v>102975.0698501281</v>
       </c>
     </row>
     <row r="333" spans="1:6">
@@ -7308,16 +7308,16 @@
         <v>2044</v>
       </c>
       <c r="C333">
-        <v>0</v>
+        <v>102522.7211616277</v>
       </c>
       <c r="D333">
         <v>0</v>
       </c>
       <c r="E333">
-        <v>0</v>
+        <v>102522.7211616277</v>
       </c>
       <c r="F333">
-        <v>0</v>
+        <v>102522.7211616277</v>
       </c>
     </row>
     <row r="334" spans="1:6">
@@ -7328,16 +7328,16 @@
         <v>2045</v>
       </c>
       <c r="C334">
-        <v>0</v>
+        <v>98538.22313310886</v>
       </c>
       <c r="D334">
         <v>0</v>
       </c>
       <c r="E334">
-        <v>0</v>
+        <v>98538.22313310886</v>
       </c>
       <c r="F334">
-        <v>0</v>
+        <v>98538.22313310886</v>
       </c>
     </row>
     <row r="335" spans="1:6">
@@ -7348,16 +7348,16 @@
         <v>2046</v>
       </c>
       <c r="C335">
-        <v>0</v>
+        <v>97057.34503861617</v>
       </c>
       <c r="D335">
         <v>0</v>
       </c>
       <c r="E335">
-        <v>0</v>
+        <v>97057.34503861617</v>
       </c>
       <c r="F335">
-        <v>0</v>
+        <v>97057.34503861617</v>
       </c>
     </row>
     <row r="336" spans="1:6">
@@ -7368,16 +7368,16 @@
         <v>2047</v>
       </c>
       <c r="C336">
-        <v>0</v>
+        <v>99266.35475068688</v>
       </c>
       <c r="D336">
         <v>0</v>
       </c>
       <c r="E336">
-        <v>0</v>
+        <v>99266.35475068688</v>
       </c>
       <c r="F336">
-        <v>0</v>
+        <v>99266.35475068688</v>
       </c>
     </row>
     <row r="337" spans="1:6">
@@ -7388,16 +7388,16 @@
         <v>2048</v>
       </c>
       <c r="C337">
-        <v>0</v>
+        <v>101276.2820638496</v>
       </c>
       <c r="D337">
         <v>0</v>
       </c>
       <c r="E337">
-        <v>0</v>
+        <v>101276.2820638496</v>
       </c>
       <c r="F337">
-        <v>0</v>
+        <v>101276.2820638496</v>
       </c>
     </row>
     <row r="338" spans="1:6">
@@ -7408,16 +7408,16 @@
         <v>2049</v>
       </c>
       <c r="C338">
-        <v>0</v>
+        <v>96149.87974452588</v>
       </c>
       <c r="D338">
         <v>0</v>
       </c>
       <c r="E338">
-        <v>0</v>
+        <v>96149.87974452588</v>
       </c>
       <c r="F338">
-        <v>0</v>
+        <v>96149.87974452588</v>
       </c>
     </row>
     <row r="339" spans="1:6">
@@ -7428,16 +7428,16 @@
         <v>2050</v>
       </c>
       <c r="C339">
-        <v>0</v>
+        <v>98186.47975212552</v>
       </c>
       <c r="D339">
         <v>0</v>
       </c>
       <c r="E339">
-        <v>0</v>
+        <v>98186.47975212552</v>
       </c>
       <c r="F339">
-        <v>0</v>
+        <v>98186.47975212552</v>
       </c>
     </row>
     <row r="340" spans="1:6">
@@ -7448,10 +7448,10 @@
         <v>2025</v>
       </c>
       <c r="C340">
-        <v>0</v>
+        <v>39326.29004948001</v>
       </c>
       <c r="D340">
-        <v>0</v>
+        <v>39326.29004948001</v>
       </c>
       <c r="E340">
         <v>0</v>
@@ -7468,13 +7468,13 @@
         <v>2026</v>
       </c>
       <c r="C341">
-        <v>0</v>
+        <v>80106.13249300426</v>
       </c>
       <c r="D341">
-        <v>0</v>
+        <v>44576.49673152481</v>
       </c>
       <c r="E341">
-        <v>0</v>
+        <v>35529.63576147945</v>
       </c>
       <c r="F341">
         <v>0</v>
@@ -7488,13 +7488,13 @@
         <v>2027</v>
       </c>
       <c r="C342">
-        <v>0</v>
+        <v>95805.55965580525</v>
       </c>
       <c r="D342">
-        <v>0</v>
+        <v>33639.634678496</v>
       </c>
       <c r="E342">
-        <v>0</v>
+        <v>62165.92497730925</v>
       </c>
       <c r="F342">
         <v>0</v>
@@ -7508,13 +7508,13 @@
         <v>2028</v>
       </c>
       <c r="C343">
-        <v>0</v>
+        <v>103225.8276081462</v>
       </c>
       <c r="D343">
-        <v>0</v>
+        <v>34404.69313785505</v>
       </c>
       <c r="E343">
-        <v>0</v>
+        <v>68821.13447029119</v>
       </c>
       <c r="F343">
         <v>0</v>
@@ -7528,13 +7528,13 @@
         <v>2029</v>
       </c>
       <c r="C344">
-        <v>0</v>
+        <v>118470.315967819</v>
       </c>
       <c r="D344">
-        <v>0</v>
+        <v>44645.74258912993</v>
       </c>
       <c r="E344">
-        <v>0</v>
+        <v>73824.57337868909</v>
       </c>
       <c r="F344">
         <v>0</v>
@@ -7548,13 +7548,13 @@
         <v>2030</v>
       </c>
       <c r="C345">
-        <v>0</v>
+        <v>127115.3682796919</v>
       </c>
       <c r="D345">
-        <v>0</v>
+        <v>40728.1798430416</v>
       </c>
       <c r="E345">
-        <v>0</v>
+        <v>86387.18843665032</v>
       </c>
       <c r="F345">
         <v>0</v>
@@ -7568,13 +7568,13 @@
         <v>2031</v>
       </c>
       <c r="C346">
-        <v>0</v>
+        <v>138995.1132540111</v>
       </c>
       <c r="D346">
-        <v>0</v>
+        <v>48169.58916535361</v>
       </c>
       <c r="E346">
-        <v>0</v>
+        <v>90825.52408865748</v>
       </c>
       <c r="F346">
         <v>0</v>
@@ -7588,13 +7588,13 @@
         <v>2032</v>
       </c>
       <c r="C347">
-        <v>0</v>
+        <v>145750.9352205967</v>
       </c>
       <c r="D347">
-        <v>0</v>
+        <v>45195.37348671073</v>
       </c>
       <c r="E347">
-        <v>0</v>
+        <v>100555.5617338859</v>
       </c>
       <c r="F347">
         <v>0</v>
@@ -7608,13 +7608,13 @@
         <v>2033</v>
       </c>
       <c r="C348">
-        <v>0</v>
+        <v>153779.1038185924</v>
       </c>
       <c r="D348">
-        <v>0</v>
+        <v>49636.85013952225</v>
       </c>
       <c r="E348">
-        <v>0</v>
+        <v>104142.2536790701</v>
       </c>
       <c r="F348">
         <v>0</v>
@@ -7628,13 +7628,13 @@
         <v>2034</v>
       </c>
       <c r="C349">
-        <v>0</v>
+        <v>153953.1847875851</v>
       </c>
       <c r="D349">
-        <v>0</v>
+        <v>43285.74394936513</v>
       </c>
       <c r="E349">
-        <v>0</v>
+        <v>110667.4408382199</v>
       </c>
       <c r="F349">
         <v>0</v>
@@ -7648,13 +7648,13 @@
         <v>2035</v>
       </c>
       <c r="C350">
-        <v>0</v>
+        <v>149980.5337310351</v>
       </c>
       <c r="D350">
-        <v>0</v>
+        <v>40725.82787864641</v>
       </c>
       <c r="E350">
-        <v>0</v>
+        <v>109254.7058523887</v>
       </c>
       <c r="F350">
         <v>0</v>
@@ -7668,13 +7668,13 @@
         <v>2036</v>
       </c>
       <c r="C351">
-        <v>0</v>
+        <v>146651.6018301565</v>
       </c>
       <c r="D351">
-        <v>0</v>
+        <v>40263.53382842337</v>
       </c>
       <c r="E351">
-        <v>0</v>
+        <v>106388.0680017331</v>
       </c>
       <c r="F351">
         <v>0</v>
@@ -7688,13 +7688,13 @@
         <v>2037</v>
       </c>
       <c r="C352">
-        <v>0</v>
+        <v>152053.4687735046</v>
       </c>
       <c r="D352">
-        <v>0</v>
+        <v>47548.58016868064</v>
       </c>
       <c r="E352">
-        <v>0</v>
+        <v>104504.888604824</v>
       </c>
       <c r="F352">
         <v>0</v>
@@ -7708,13 +7708,13 @@
         <v>2038</v>
       </c>
       <c r="C353">
-        <v>0</v>
+        <v>155709.8206907659</v>
       </c>
       <c r="D353">
-        <v>0</v>
+        <v>45502.99890641568</v>
       </c>
       <c r="E353">
-        <v>0</v>
+        <v>110206.8217843502</v>
       </c>
       <c r="F353">
         <v>0</v>
@@ -7728,13 +7728,13 @@
         <v>2039</v>
       </c>
       <c r="C354">
-        <v>0</v>
+        <v>151553.0397731369</v>
       </c>
       <c r="D354">
-        <v>0</v>
+        <v>39416.42205561985</v>
       </c>
       <c r="E354">
-        <v>0</v>
+        <v>112136.617717517</v>
       </c>
       <c r="F354">
         <v>0</v>
@@ -7748,13 +7748,13 @@
         <v>2040</v>
       </c>
       <c r="C355">
-        <v>0</v>
+        <v>156970.6800413339</v>
       </c>
       <c r="D355">
-        <v>0</v>
+        <v>48868.78828749121</v>
       </c>
       <c r="E355">
-        <v>0</v>
+        <v>108101.8917538427</v>
       </c>
       <c r="F355">
         <v>0</v>
@@ -7768,13 +7768,13 @@
         <v>2041</v>
       </c>
       <c r="C356">
-        <v>0</v>
+        <v>154273.9760511113</v>
       </c>
       <c r="D356">
-        <v>0</v>
+        <v>39846.05995828417</v>
       </c>
       <c r="E356">
-        <v>0</v>
+        <v>114427.9160928271</v>
       </c>
       <c r="F356">
         <v>0</v>
@@ -7788,13 +7788,13 @@
         <v>2042</v>
       </c>
       <c r="C357">
-        <v>0</v>
+        <v>153964.2986577101</v>
       </c>
       <c r="D357">
-        <v>0</v>
+        <v>43540.99731744001</v>
       </c>
       <c r="E357">
-        <v>0</v>
+        <v>110423.3013402701</v>
       </c>
       <c r="F357">
         <v>0</v>
@@ -7808,13 +7808,13 @@
         <v>2043</v>
       </c>
       <c r="C358">
-        <v>0</v>
+        <v>153517.0595726243</v>
       </c>
       <c r="D358">
-        <v>0</v>
+        <v>41960.73390165217</v>
       </c>
       <c r="E358">
-        <v>0</v>
+        <v>111556.3256709721</v>
       </c>
       <c r="F358">
         <v>0</v>
@@ -7828,13 +7828,13 @@
         <v>2044</v>
       </c>
       <c r="C359">
-        <v>0</v>
+        <v>148323.1050889702</v>
       </c>
       <c r="D359">
-        <v>0</v>
+        <v>37256.82383054017</v>
       </c>
       <c r="E359">
-        <v>0</v>
+        <v>111066.28125843</v>
       </c>
       <c r="F359">
         <v>0</v>
@@ -7848,13 +7848,13 @@
         <v>2045</v>
       </c>
       <c r="C360">
-        <v>0</v>
+        <v>144925.360130493</v>
       </c>
       <c r="D360">
-        <v>0</v>
+        <v>38175.61840295841</v>
       </c>
       <c r="E360">
-        <v>0</v>
+        <v>106749.7417275346</v>
       </c>
       <c r="F360">
         <v>0</v>
@@ -7868,13 +7868,13 @@
         <v>2046</v>
       </c>
       <c r="C361">
-        <v>0</v>
+        <v>146839.6958505739</v>
       </c>
       <c r="D361">
-        <v>0</v>
+        <v>41694.23872540641</v>
       </c>
       <c r="E361">
-        <v>0</v>
+        <v>105145.4571251675</v>
       </c>
       <c r="F361">
         <v>0</v>
@@ -7888,13 +7888,13 @@
         <v>2047</v>
       </c>
       <c r="C362">
-        <v>0</v>
+        <v>149800.2100468657</v>
       </c>
       <c r="D362">
-        <v>0</v>
+        <v>42261.65906695489</v>
       </c>
       <c r="E362">
-        <v>0</v>
+        <v>107538.5509799108</v>
       </c>
       <c r="F362">
         <v>0</v>
@@ -7908,13 +7908,13 @@
         <v>2048</v>
       </c>
       <c r="C363">
-        <v>0</v>
+        <v>144133.0394498838</v>
       </c>
       <c r="D363">
-        <v>0</v>
+        <v>34417.06721404673</v>
       </c>
       <c r="E363">
-        <v>0</v>
+        <v>109715.9722358371</v>
       </c>
       <c r="F363">
         <v>0</v>
@@ -7928,13 +7928,13 @@
         <v>2049</v>
       </c>
       <c r="C364">
-        <v>0</v>
+        <v>144595.7364125772</v>
       </c>
       <c r="D364">
-        <v>0</v>
+        <v>40433.3666893408</v>
       </c>
       <c r="E364">
-        <v>0</v>
+        <v>104162.3697232364</v>
       </c>
       <c r="F364">
         <v>0</v>
@@ -7948,13 +7948,13 @@
         <v>2050</v>
       </c>
       <c r="C365">
-        <v>0</v>
+        <v>145918.808232128</v>
       </c>
       <c r="D365">
-        <v>0</v>
+        <v>39550.12183399201</v>
       </c>
       <c r="E365">
-        <v>0</v>
+        <v>106368.686398136</v>
       </c>
       <c r="F365">
         <v>0</v>
@@ -8018,16 +8018,16 @@
         <v>2026</v>
       </c>
       <c r="C3">
-        <v>-131436.9879283817</v>
+        <v>-98640.40107163147</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="E3">
-        <v>-131436.9879283817</v>
+        <v>-98640.40107163147</v>
       </c>
       <c r="F3">
-        <v>-131436.9879283817</v>
+        <v>-98640.40107163147</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -8038,16 +8038,16 @@
         <v>2027</v>
       </c>
       <c r="C4">
-        <v>-99188.8684805939</v>
+        <v>-41804.93773230843</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>-99188.8684805939</v>
+        <v>-41804.93773230843</v>
       </c>
       <c r="F4">
-        <v>-99188.8684805939</v>
+        <v>-41804.93773230843</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -8058,16 +8058,16 @@
         <v>2028</v>
       </c>
       <c r="C5">
-        <v>-101444.6952430469</v>
+        <v>-37917.49419354729</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>-101444.6952430469</v>
+        <v>-37917.49419354729</v>
       </c>
       <c r="F5">
-        <v>-101444.6952430469</v>
+        <v>-37917.49419354729</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -8078,16 +8078,16 @@
         <v>2029</v>
       </c>
       <c r="C6">
-        <v>-131641.1611336631</v>
+        <v>-63495.40109179623</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6">
-        <v>-131641.1611336631</v>
+        <v>-63495.40109179623</v>
       </c>
       <c r="F6">
-        <v>-131641.1611336631</v>
+        <v>-63495.40109179623</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -8098,16 +8098,16 @@
         <v>2030</v>
       </c>
       <c r="C7">
-        <v>-120089.9450549113</v>
+        <v>-40347.92495954176</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>-120089.9450549113</v>
+        <v>-40347.92495954176</v>
       </c>
       <c r="F7">
-        <v>-120089.9450549113</v>
+        <v>-40347.92495954176</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -8118,16 +8118,16 @@
         <v>2031</v>
       </c>
       <c r="C8">
-        <v>-142031.4744989855</v>
+        <v>-58192.52918637858</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>-142031.4744989855</v>
+        <v>-58192.52918637858</v>
       </c>
       <c r="F8">
-        <v>-142031.4744989855</v>
+        <v>-58192.52918637858</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -8138,16 +8138,16 @@
         <v>2032</v>
       </c>
       <c r="C9">
-        <v>-133261.7868225299</v>
+        <v>-40441.26829894294</v>
       </c>
       <c r="D9">
         <v>0</v>
       </c>
       <c r="E9">
-        <v>-133261.7868225299</v>
+        <v>-40441.26829894294</v>
       </c>
       <c r="F9">
-        <v>-133261.7868225299</v>
+        <v>-40441.26829894294</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -8158,16 +8158,16 @@
         <v>2033</v>
       </c>
       <c r="C10">
-        <v>-146357.795133677</v>
+        <v>-50226.48404530459</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10">
-        <v>-146357.795133677</v>
+        <v>-50226.48404530459</v>
       </c>
       <c r="F10">
-        <v>-146357.795133677</v>
+        <v>-50226.48404530459</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -8178,16 +8178,16 @@
         <v>2034</v>
       </c>
       <c r="C11">
-        <v>-127631.1071215566</v>
+        <v>-25476.54634781508</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>-127631.1071215566</v>
+        <v>-25476.54634781508</v>
       </c>
       <c r="F11">
-        <v>-127631.1071215566</v>
+        <v>-25476.54634781508</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -8198,16 +8198,16 @@
         <v>2035</v>
       </c>
       <c r="C12">
-        <v>-120083.0104718946</v>
+        <v>-19232.51276199729</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12">
-        <v>-120083.0104718946</v>
+        <v>-19232.51276199729</v>
       </c>
       <c r="F12">
-        <v>-120083.0104718946</v>
+        <v>-19232.51276199729</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -8218,16 +8218,16 @@
         <v>2036</v>
       </c>
       <c r="C13">
-        <v>-118719.9049958083</v>
+        <v>-20515.53453267011</v>
       </c>
       <c r="D13">
         <v>0</v>
       </c>
       <c r="E13">
-        <v>-118719.9049958083</v>
+        <v>-20515.53453267011</v>
       </c>
       <c r="F13">
-        <v>-118719.9049958083</v>
+        <v>-20515.53453267011</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -8238,16 +8238,16 @@
         <v>2037</v>
       </c>
       <c r="C14">
-        <v>-140200.3815465098</v>
+        <v>-43734.3305266723</v>
       </c>
       <c r="D14">
         <v>0</v>
       </c>
       <c r="E14">
-        <v>-140200.3815465098</v>
+        <v>-43734.3305266723</v>
       </c>
       <c r="F14">
-        <v>-140200.3815465098</v>
+        <v>-43734.3305266723</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -8258,16 +8258,16 @@
         <v>2038</v>
       </c>
       <c r="C15">
-        <v>-134168.8429857742</v>
+        <v>-32439.46903098945</v>
       </c>
       <c r="D15">
         <v>0</v>
       </c>
       <c r="E15">
-        <v>-134168.8429857742</v>
+        <v>-32439.46903098945</v>
       </c>
       <c r="F15">
-        <v>-134168.8429857742</v>
+        <v>-32439.46903098945</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -8278,16 +8278,16 @@
         <v>2039</v>
       </c>
       <c r="C16">
-        <v>-116222.1351057133</v>
+        <v>-12711.41105877457</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <v>-116222.1351057133</v>
+        <v>-12711.41105877457</v>
       </c>
       <c r="F16">
-        <v>-116222.1351057133</v>
+        <v>-12711.41105877457</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -8298,16 +8298,16 @@
         <v>2040</v>
       </c>
       <c r="C17">
-        <v>-144093.1122214027</v>
+        <v>-44306.75060247094</v>
       </c>
       <c r="D17">
         <v>0</v>
       </c>
       <c r="E17">
-        <v>-144093.1122214027</v>
+        <v>-44306.75060247094</v>
       </c>
       <c r="F17">
-        <v>-144093.1122214027</v>
+        <v>-44306.75060247094</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -8318,16 +8318,16 @@
         <v>2041</v>
       </c>
       <c r="C18">
-        <v>-117488.9546701407</v>
+        <v>-11863.18596906948</v>
       </c>
       <c r="D18">
         <v>0</v>
       </c>
       <c r="E18">
-        <v>-117488.9546701407</v>
+        <v>-11863.18596906948</v>
       </c>
       <c r="F18">
-        <v>-117488.9546701407</v>
+        <v>-11863.18596906948</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -8338,16 +8338,16 @@
         <v>2042</v>
       </c>
       <c r="C19">
-        <v>-128383.7426617088</v>
+        <v>-26454.54142453638</v>
       </c>
       <c r="D19">
         <v>0</v>
       </c>
       <c r="E19">
-        <v>-128383.7426617088</v>
+        <v>-26454.54142453638</v>
       </c>
       <c r="F19">
-        <v>-128383.7426617088</v>
+        <v>-26454.54142453638</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -8358,16 +8358,16 @@
         <v>2043</v>
       </c>
       <c r="C20">
-        <v>-123724.2235363001</v>
+        <v>-20749.15368617198</v>
       </c>
       <c r="D20">
         <v>0</v>
       </c>
       <c r="E20">
-        <v>-123724.2235363001</v>
+        <v>-20749.15368617198</v>
       </c>
       <c r="F20">
-        <v>-123724.2235363001</v>
+        <v>-20749.15368617198</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -8378,16 +8378,16 @@
         <v>2044</v>
       </c>
       <c r="C21">
-        <v>-109854.4073700498</v>
+        <v>-7331.686208422121</v>
       </c>
       <c r="D21">
         <v>0</v>
       </c>
       <c r="E21">
-        <v>-109854.4073700498</v>
+        <v>-7331.686208422121</v>
       </c>
       <c r="F21">
-        <v>-109854.4073700498</v>
+        <v>-7331.686208422121</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -8398,16 +8398,16 @@
         <v>2045</v>
       </c>
       <c r="C22">
-        <v>-112563.5405230088</v>
+        <v>-14025.31738989992</v>
       </c>
       <c r="D22">
         <v>0</v>
       </c>
       <c r="E22">
-        <v>-112563.5405230088</v>
+        <v>-14025.31738989992</v>
       </c>
       <c r="F22">
-        <v>-112563.5405230088</v>
+        <v>-14025.31738989992</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -8418,16 +8418,16 @@
         <v>2046</v>
       </c>
       <c r="C23">
-        <v>-122938.4412817697</v>
+        <v>-25881.09624315356</v>
       </c>
       <c r="D23">
         <v>0</v>
       </c>
       <c r="E23">
-        <v>-122938.4412817697</v>
+        <v>-25881.09624315356</v>
       </c>
       <c r="F23">
-        <v>-122938.4412817697</v>
+        <v>-25881.09624315356</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -8438,16 +8438,16 @@
         <v>2047</v>
       </c>
       <c r="C24">
-        <v>-124611.5205928498</v>
+        <v>-25345.16584216297</v>
       </c>
       <c r="D24">
         <v>0</v>
       </c>
       <c r="E24">
-        <v>-124611.5205928498</v>
+        <v>-25345.16584216297</v>
       </c>
       <c r="F24">
-        <v>-124611.5205928498</v>
+        <v>-25345.16584216297</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -8458,16 +8458,16 @@
         <v>2048</v>
       </c>
       <c r="C25">
-        <v>-101481.1837465606</v>
+        <v>-204.9016827109735</v>
       </c>
       <c r="D25">
         <v>0</v>
       </c>
       <c r="E25">
-        <v>-101481.1837465606</v>
+        <v>-204.9016827109735</v>
       </c>
       <c r="F25">
-        <v>-101481.1837465606</v>
+        <v>-204.9016827109735</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -8478,16 +8478,16 @@
         <v>2049</v>
       </c>
       <c r="C26">
-        <v>-119220.668901142</v>
+        <v>-23070.78915661614</v>
       </c>
       <c r="D26">
         <v>0</v>
       </c>
       <c r="E26">
-        <v>-119220.668901142</v>
+        <v>-23070.78915661614</v>
       </c>
       <c r="F26">
-        <v>-119220.668901142</v>
+        <v>-23070.78915661614</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -8498,16 +8498,16 @@
         <v>2050</v>
       </c>
       <c r="C27">
-        <v>-116616.3586122278</v>
+        <v>-18429.87886010227</v>
       </c>
       <c r="D27">
         <v>0</v>
       </c>
       <c r="E27">
-        <v>-116616.3586122278</v>
+        <v>-18429.87886010227</v>
       </c>
       <c r="F27">
-        <v>-116616.3586122278</v>
+        <v>-18429.87886010227</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -8558,16 +8558,16 @@
         <v>2027</v>
       </c>
       <c r="C30">
-        <v>-247393.3621199913</v>
+        <v>-214596.7752632411</v>
       </c>
       <c r="D30">
         <v>0</v>
       </c>
       <c r="E30">
-        <v>-247393.3621199913</v>
+        <v>-214596.7752632411</v>
       </c>
       <c r="F30">
-        <v>-247393.3621199913</v>
+        <v>-214596.7752632411</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -8578,16 +8578,16 @@
         <v>2028</v>
       </c>
       <c r="C31">
-        <v>-346582.2306005852</v>
+        <v>-256401.7129955495</v>
       </c>
       <c r="D31">
         <v>0</v>
       </c>
       <c r="E31">
-        <v>-346582.2306005852</v>
+        <v>-256401.7129955495</v>
       </c>
       <c r="F31">
-        <v>-346582.2306005852</v>
+        <v>-256401.7129955495</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -8598,16 +8598,16 @@
         <v>2029</v>
       </c>
       <c r="C32">
-        <v>-448026.9258436321</v>
+        <v>-294319.2071890968</v>
       </c>
       <c r="D32">
         <v>0</v>
       </c>
       <c r="E32">
-        <v>-448026.9258436321</v>
+        <v>-294319.2071890968</v>
       </c>
       <c r="F32">
-        <v>-448026.9258436321</v>
+        <v>-294319.2071890968</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -8618,16 +8618,16 @@
         <v>2030</v>
       </c>
       <c r="C33">
-        <v>-579668.0869772951</v>
+        <v>-357814.6082808931</v>
       </c>
       <c r="D33">
         <v>0</v>
       </c>
       <c r="E33">
-        <v>-579668.0869772951</v>
+        <v>-357814.6082808931</v>
       </c>
       <c r="F33">
-        <v>-579668.0869772951</v>
+        <v>-357814.6082808931</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -8638,16 +8638,16 @@
         <v>2031</v>
       </c>
       <c r="C34">
-        <v>-699758.0320322064</v>
+        <v>-398162.5332404348</v>
       </c>
       <c r="D34">
         <v>0</v>
       </c>
       <c r="E34">
-        <v>-699758.0320322064</v>
+        <v>-398162.5332404348</v>
       </c>
       <c r="F34">
-        <v>-699758.0320322064</v>
+        <v>-398162.5332404348</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -8658,16 +8658,16 @@
         <v>2032</v>
       </c>
       <c r="C35">
-        <v>-841789.5065311919</v>
+        <v>-456355.0624268134</v>
       </c>
       <c r="D35">
         <v>0</v>
       </c>
       <c r="E35">
-        <v>-841789.5065311919</v>
+        <v>-456355.0624268134</v>
       </c>
       <c r="F35">
-        <v>-841789.5065311919</v>
+        <v>-456355.0624268134</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -8678,16 +8678,16 @@
         <v>2033</v>
       </c>
       <c r="C36">
-        <v>-975051.2933537217</v>
+        <v>-496796.3307257564</v>
       </c>
       <c r="D36">
         <v>0</v>
       </c>
       <c r="E36">
-        <v>-975051.2933537217</v>
+        <v>-496796.3307257564</v>
       </c>
       <c r="F36">
-        <v>-975051.2933537217</v>
+        <v>-496796.3307257564</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -8698,16 +8698,16 @@
         <v>2034</v>
       </c>
       <c r="C37">
-        <v>-1121409.088487399</v>
+        <v>-547022.8147710609</v>
       </c>
       <c r="D37">
         <v>0</v>
       </c>
       <c r="E37">
-        <v>-1121409.088487399</v>
+        <v>-547022.8147710609</v>
       </c>
       <c r="F37">
-        <v>-1121409.088487399</v>
+        <v>-547022.8147710609</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -8718,16 +8718,16 @@
         <v>2035</v>
       </c>
       <c r="C38">
-        <v>-1249040.195608955</v>
+        <v>-572499.361118876</v>
       </c>
       <c r="D38">
         <v>0</v>
       </c>
       <c r="E38">
-        <v>-1249040.195608955</v>
+        <v>-572499.361118876</v>
       </c>
       <c r="F38">
-        <v>-1249040.195608955</v>
+        <v>-572499.361118876</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -8738,16 +8738,16 @@
         <v>2036</v>
       </c>
       <c r="C39">
-        <v>-1369123.20608085</v>
+        <v>-591731.8738808733</v>
       </c>
       <c r="D39">
         <v>0</v>
       </c>
       <c r="E39">
-        <v>-1369123.20608085</v>
+        <v>-591731.8738808733</v>
       </c>
       <c r="F39">
-        <v>-1369123.20608085</v>
+        <v>-591731.8738808733</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -8758,16 +8758,16 @@
         <v>2037</v>
       </c>
       <c r="C40">
-        <v>-1487843.111076658</v>
+        <v>-612247.4084135434</v>
       </c>
       <c r="D40">
         <v>0</v>
       </c>
       <c r="E40">
-        <v>-1487843.111076658</v>
+        <v>-612247.4084135434</v>
       </c>
       <c r="F40">
-        <v>-1487843.111076658</v>
+        <v>-612247.4084135434</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -8778,16 +8778,16 @@
         <v>2038</v>
       </c>
       <c r="C41">
-        <v>-1628043.492623168</v>
+        <v>-655981.7389402157</v>
       </c>
       <c r="D41">
         <v>0</v>
       </c>
       <c r="E41">
-        <v>-1628043.492623168</v>
+        <v>-655981.7389402157</v>
       </c>
       <c r="F41">
-        <v>-1628043.492623168</v>
+        <v>-655981.7389402157</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -8798,16 +8798,16 @@
         <v>2039</v>
       </c>
       <c r="C42">
-        <v>-1762212.335608942</v>
+        <v>-688421.2079712051</v>
       </c>
       <c r="D42">
         <v>0</v>
       </c>
       <c r="E42">
-        <v>-1762212.335608942</v>
+        <v>-688421.2079712051</v>
       </c>
       <c r="F42">
-        <v>-1762212.335608942</v>
+        <v>-688421.2079712051</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -8818,16 +8818,16 @@
         <v>2040</v>
       </c>
       <c r="C43">
-        <v>-1878434.470714655</v>
+        <v>-701132.6190299797</v>
       </c>
       <c r="D43">
         <v>0</v>
       </c>
       <c r="E43">
-        <v>-1878434.470714655</v>
+        <v>-701132.6190299797</v>
       </c>
       <c r="F43">
-        <v>-1878434.470714655</v>
+        <v>-701132.6190299797</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -8838,16 +8838,16 @@
         <v>2041</v>
       </c>
       <c r="C44">
-        <v>-2022527.582936058</v>
+        <v>-745439.3696324506</v>
       </c>
       <c r="D44">
         <v>0</v>
       </c>
       <c r="E44">
-        <v>-2022527.582936058</v>
+        <v>-745439.3696324506</v>
       </c>
       <c r="F44">
-        <v>-2022527.582936058</v>
+        <v>-745439.3696324506</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -8858,16 +8858,16 @@
         <v>2042</v>
       </c>
       <c r="C45">
-        <v>-2140016.537606199</v>
+        <v>-757302.5556015201</v>
       </c>
       <c r="D45">
         <v>0</v>
       </c>
       <c r="E45">
-        <v>-2140016.537606199</v>
+        <v>-757302.5556015201</v>
       </c>
       <c r="F45">
-        <v>-2140016.537606199</v>
+        <v>-757302.5556015201</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -8878,16 +8878,16 @@
         <v>2043</v>
       </c>
       <c r="C46">
-        <v>-2268400.280267908</v>
+        <v>-783757.0970260565</v>
       </c>
       <c r="D46">
         <v>0</v>
       </c>
       <c r="E46">
-        <v>-2268400.280267908</v>
+        <v>-783757.0970260565</v>
       </c>
       <c r="F46">
-        <v>-2268400.280267908</v>
+        <v>-783757.0970260565</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -8898,16 +8898,16 @@
         <v>2044</v>
       </c>
       <c r="C47">
-        <v>-2392124.503804208</v>
+        <v>-804506.2507122285</v>
       </c>
       <c r="D47">
         <v>0</v>
       </c>
       <c r="E47">
-        <v>-2392124.503804208</v>
+        <v>-804506.2507122285</v>
       </c>
       <c r="F47">
-        <v>-2392124.503804208</v>
+        <v>-804506.2507122285</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -8918,16 +8918,16 @@
         <v>2045</v>
       </c>
       <c r="C48">
-        <v>-2501978.911174258</v>
+        <v>-811837.9369206505</v>
       </c>
       <c r="D48">
         <v>0</v>
       </c>
       <c r="E48">
-        <v>-2501978.911174258</v>
+        <v>-811837.9369206505</v>
       </c>
       <c r="F48">
-        <v>-2501978.911174258</v>
+        <v>-811837.9369206505</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -8938,16 +8938,16 @@
         <v>2046</v>
       </c>
       <c r="C49">
-        <v>-2614542.451697267</v>
+        <v>-825863.2543105504</v>
       </c>
       <c r="D49">
         <v>0</v>
       </c>
       <c r="E49">
-        <v>-2614542.451697267</v>
+        <v>-825863.2543105504</v>
       </c>
       <c r="F49">
-        <v>-2614542.451697267</v>
+        <v>-825863.2543105504</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -8958,16 +8958,16 @@
         <v>2047</v>
       </c>
       <c r="C50">
-        <v>-2737480.892979037</v>
+        <v>-851744.350553704</v>
       </c>
       <c r="D50">
         <v>0</v>
       </c>
       <c r="E50">
-        <v>-2737480.892979037</v>
+        <v>-851744.350553704</v>
       </c>
       <c r="F50">
-        <v>-2737480.892979037</v>
+        <v>-851744.350553704</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -8978,16 +8978,16 @@
         <v>2048</v>
       </c>
       <c r="C51">
-        <v>-2862092.413571886</v>
+        <v>-877089.5163958669</v>
       </c>
       <c r="D51">
         <v>0</v>
       </c>
       <c r="E51">
-        <v>-2862092.413571886</v>
+        <v>-877089.5163958669</v>
       </c>
       <c r="F51">
-        <v>-2862092.413571886</v>
+        <v>-877089.5163958669</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -8998,16 +8998,16 @@
         <v>2049</v>
       </c>
       <c r="C52">
-        <v>-2963573.597318447</v>
+        <v>-877294.4180785778</v>
       </c>
       <c r="D52">
         <v>0</v>
       </c>
       <c r="E52">
-        <v>-2963573.597318447</v>
+        <v>-877294.4180785778</v>
       </c>
       <c r="F52">
-        <v>-2963573.597318447</v>
+        <v>-877294.4180785778</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -9018,16 +9018,16 @@
         <v>2050</v>
       </c>
       <c r="C53">
-        <v>-3082794.266219589</v>
+        <v>-900365.207235194</v>
       </c>
       <c r="D53">
         <v>0</v>
       </c>
       <c r="E53">
-        <v>-3082794.266219589</v>
+        <v>-900365.207235194</v>
       </c>
       <c r="F53">
-        <v>-3082794.266219589</v>
+        <v>-900365.207235194</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -9038,10 +9038,10 @@
         <v>2025</v>
       </c>
       <c r="C54">
-        <v>-164945.6975903904</v>
+        <v>-125619.4075409104</v>
       </c>
       <c r="D54">
-        <v>-39326.29020092187</v>
+        <v>-0.00015144185454119</v>
       </c>
       <c r="E54">
         <v>-125619.4073894685</v>
@@ -9058,13 +9058,13 @@
         <v>2026</v>
       </c>
       <c r="C55">
-        <v>-186966.5601539384</v>
+        <v>-106860.4276609341</v>
       </c>
       <c r="D55">
-        <v>-44576.49584010887</v>
+        <v>0.0008914159407140687</v>
       </c>
       <c r="E55">
-        <v>-142390.0643138295</v>
+        <v>-106860.42855235</v>
       </c>
       <c r="F55">
         <v>0</v>
@@ -9078,13 +9078,13 @@
         <v>2027</v>
       </c>
       <c r="C56">
-        <v>-141094.2363658061</v>
+        <v>-45288.67671000079</v>
       </c>
       <c r="D56">
-        <v>-33639.63392836272</v>
+        <v>0.0007501333020627499</v>
       </c>
       <c r="E56">
-        <v>-107454.6024374434</v>
+        <v>-45288.67746013409</v>
       </c>
       <c r="F56">
         <v>0</v>
@@ -9098,13 +9098,13 @@
         <v>2028</v>
       </c>
       <c r="C57">
-        <v>-144303.1128844892</v>
+        <v>-41077.28527634294</v>
       </c>
       <c r="D57">
-        <v>-34404.69304197494</v>
+        <v>9.588011016603559E-05</v>
       </c>
       <c r="E57">
-        <v>-109898.4198425142</v>
+        <v>-41077.28537222301</v>
       </c>
       <c r="F57">
         <v>0</v>
@@ -9118,13 +9118,13 @@
         <v>2029</v>
       </c>
       <c r="C58">
-        <v>-187257.000217265</v>
+        <v>-68786.68424944597</v>
       </c>
       <c r="D58">
-        <v>-44645.74244904269</v>
+        <v>0.0001400872424710542</v>
       </c>
       <c r="E58">
-        <v>-142611.2577682223</v>
+        <v>-68786.68438953318</v>
       </c>
       <c r="F58">
         <v>0</v>
@@ -9138,13 +9138,13 @@
         <v>2030</v>
       </c>
       <c r="C59">
-        <v>-170825.6252525288</v>
+        <v>-43710.25697283685</v>
       </c>
       <c r="D59">
-        <v>-40728.1803076642</v>
+        <v>-0.0004646225861506537</v>
       </c>
       <c r="E59">
-        <v>-130097.4449448646</v>
+        <v>-43710.25650821428</v>
       </c>
       <c r="F59">
         <v>0</v>
@@ -9158,13 +9158,13 @@
         <v>2031</v>
       </c>
       <c r="C60">
-        <v>-202037.0195392545</v>
+        <v>-63041.90628524346</v>
       </c>
       <c r="D60">
-        <v>-48169.58900898871</v>
+        <v>0.0001563648984301835</v>
       </c>
       <c r="E60">
-        <v>-153867.4305302658</v>
+        <v>-63041.90644160839</v>
       </c>
       <c r="F60">
         <v>0</v>
@@ -9178,13 +9178,13 @@
         <v>2032</v>
       </c>
       <c r="C61">
-        <v>-189562.3095111181</v>
+        <v>-43811.37429052143</v>
       </c>
       <c r="D61">
-        <v>-45195.37341012471</v>
+        <v>7.658601680304855E-05</v>
       </c>
       <c r="E61">
-        <v>-144366.9361009934</v>
+        <v>-43811.37436710746</v>
       </c>
       <c r="F61">
         <v>0</v>
@@ -9198,13 +9198,13 @@
         <v>2033</v>
       </c>
       <c r="C62">
-        <v>-208191.134434339</v>
+        <v>-54412.03061574663</v>
       </c>
       <c r="D62">
-        <v>-49636.85073105502</v>
+        <v>-0.0005915327637922019</v>
       </c>
       <c r="E62">
-        <v>-158554.283703284</v>
+        <v>-54412.03002421389</v>
       </c>
       <c r="F62">
         <v>0</v>
@@ -9218,13 +9218,13 @@
         <v>2034</v>
       </c>
       <c r="C63">
-        <v>-181552.7782310514</v>
+        <v>-27599.59344346635</v>
       </c>
       <c r="D63">
-        <v>-43285.74402242484</v>
+        <v>-7.305970939341933E-05</v>
       </c>
       <c r="E63">
-        <v>-138267.0342086266</v>
+        <v>-27599.59337040666</v>
       </c>
       <c r="F63">
         <v>0</v>
@@ -9238,13 +9238,13 @@
         <v>2035</v>
       </c>
       <c r="C64">
-        <v>-170815.7600898655</v>
+        <v>-20835.2263588304</v>
       </c>
       <c r="D64">
-        <v>-40725.82825935107</v>
+        <v>-0.0003807046596193686</v>
       </c>
       <c r="E64">
-        <v>-130089.9318305145</v>
+        <v>-20835.22597812576</v>
       </c>
       <c r="F64">
         <v>0</v>
@@ -9258,13 +9258,13 @@
         <v>2036</v>
       </c>
       <c r="C65">
-        <v>-168876.7652072157</v>
+        <v>-22225.16337705927</v>
       </c>
       <c r="D65">
-        <v>-40263.53384023535</v>
+        <v>-1.181197876576334E-05</v>
       </c>
       <c r="E65">
-        <v>-128613.2313669804</v>
+        <v>-22225.16336524725</v>
       </c>
       <c r="F65">
         <v>0</v>
@@ -9278,13 +9278,13 @@
         <v>2037</v>
       </c>
       <c r="C66">
-        <v>-199432.3339440663</v>
+        <v>-47378.86517056165</v>
       </c>
       <c r="D66">
-        <v>-47548.58086452102</v>
+        <v>-0.0006958403828321025</v>
       </c>
       <c r="E66">
-        <v>-151883.7530795452</v>
+        <v>-47378.86447472125</v>
       </c>
       <c r="F66">
         <v>0</v>
@@ -9298,13 +9298,13 @@
         <v>2038</v>
       </c>
       <c r="C67">
-        <v>-190852.5777743378</v>
+        <v>-35142.75708357192</v>
       </c>
       <c r="D67">
-        <v>-45502.99867648614</v>
+        <v>0.000229929544730112</v>
       </c>
       <c r="E67">
-        <v>-145349.5790978516</v>
+        <v>-35142.75731350138</v>
       </c>
       <c r="F67">
         <v>0</v>
@@ -9318,13 +9318,13 @@
         <v>2039</v>
       </c>
       <c r="C68">
-        <v>-165323.7367201426</v>
+        <v>-13770.69694700575</v>
       </c>
       <c r="D68">
-        <v>-39416.42214580506</v>
+        <v>-9.018521814141423E-05</v>
       </c>
       <c r="E68">
-        <v>-125907.3145743376</v>
+        <v>-13770.69685682055</v>
       </c>
       <c r="F68">
         <v>0</v>
@@ -9338,13 +9338,13 @@
         <v>2040</v>
       </c>
       <c r="C69">
-        <v>-204969.6612606774</v>
+        <v>-47998.98121934349</v>
       </c>
       <c r="D69">
-        <v>-48868.78832777544</v>
+        <v>-4.028421244584024E-05</v>
       </c>
       <c r="E69">
-        <v>-156100.872932902</v>
+        <v>-47998.98117905925</v>
       </c>
       <c r="F69">
         <v>0</v>
@@ -9358,13 +9358,13 @@
         <v>2041</v>
       </c>
       <c r="C70">
-        <v>-167125.7593176033</v>
+        <v>-12851.78326649201</v>
       </c>
       <c r="D70">
-        <v>-39846.05968501716</v>
+        <v>0.0002732670109253377</v>
       </c>
       <c r="E70">
-        <v>-127279.6996325861</v>
+        <v>-12851.783539759</v>
       </c>
       <c r="F70">
         <v>0</v>
@@ -9378,13 +9378,13 @@
         <v>2042</v>
       </c>
       <c r="C71">
-        <v>-182623.3810342913</v>
+        <v>-28659.08237658109</v>
       </c>
       <c r="D71">
-        <v>-43540.9967337425</v>
+        <v>0.0005836975033162162</v>
       </c>
       <c r="E71">
-        <v>-139082.3843005488</v>
+        <v>-28659.08296027867</v>
       </c>
       <c r="F71">
         <v>0</v>
@@ -9398,13 +9398,13 @@
         <v>2043</v>
       </c>
       <c r="C72">
-        <v>-175995.3043326439</v>
+        <v>-22478.24476001959</v>
       </c>
       <c r="D72">
-        <v>-41960.73321883565</v>
+        <v>0.0006828165205661207</v>
       </c>
       <c r="E72">
-        <v>-134034.5711138083</v>
+        <v>-22478.24544283608</v>
       </c>
       <c r="F72">
         <v>0</v>
@@ -9418,13 +9418,13 @@
         <v>2044</v>
       </c>
       <c r="C73">
-        <v>-156265.7628480942</v>
+        <v>-7942.657759124006</v>
       </c>
       <c r="D73">
-        <v>-37256.82347588925</v>
+        <v>0.0003546509105945006</v>
       </c>
       <c r="E73">
-        <v>-119008.9393722049</v>
+        <v>-7942.658113774902</v>
       </c>
       <c r="F73">
         <v>0</v>
@@ -9438,13 +9438,13 @@
         <v>2045</v>
       </c>
       <c r="C74">
-        <v>-160119.4480695512</v>
+        <v>-15194.0879390582</v>
       </c>
       <c r="D74">
-        <v>-38175.61763406348</v>
+        <v>0.000768894940847531</v>
       </c>
       <c r="E74">
-        <v>-121943.8304354877</v>
+        <v>-15194.08870795311</v>
       </c>
       <c r="F74">
         <v>0</v>
@@ -9458,13 +9458,13 @@
         <v>2046</v>
       </c>
       <c r="C75">
-        <v>-174877.5496139904</v>
+        <v>-28037.85376341635</v>
       </c>
       <c r="D75">
-        <v>-41694.23856585975</v>
+        <v>0.0001595466746948659</v>
       </c>
       <c r="E75">
-        <v>-133183.3110481306</v>
+        <v>-28037.85392296308</v>
       </c>
       <c r="F75">
         <v>0</v>
@@ -9478,13 +9478,13 @@
         <v>2047</v>
       </c>
       <c r="C76">
-        <v>-177257.4727425422</v>
+        <v>-27457.26269567653</v>
       </c>
       <c r="D76">
-        <v>-42261.65892890394</v>
+        <v>0.0001380509493174031</v>
       </c>
       <c r="E76">
-        <v>-134995.8138136383</v>
+        <v>-27457.26283372747</v>
       </c>
       <c r="F76">
         <v>0</v>
@@ -9498,13 +9498,13 @@
         <v>2048</v>
       </c>
       <c r="C77">
-        <v>-144355.0106394874</v>
+        <v>-221.9711896035587</v>
       </c>
       <c r="D77">
-        <v>-34417.06648489375</v>
+        <v>0.0007291529764188454</v>
       </c>
       <c r="E77">
-        <v>-109937.9441545937</v>
+        <v>-221.9719187565497</v>
       </c>
       <c r="F77">
         <v>0</v>
@@ -9518,13 +9518,13 @@
         <v>2049</v>
       </c>
       <c r="C78">
-        <v>-169589.093165578</v>
+        <v>-24993.35675300081</v>
       </c>
       <c r="D78">
-        <v>-40433.36679991853</v>
+        <v>-0.0001105777337215841</v>
       </c>
       <c r="E78">
-        <v>-129155.7263656595</v>
+        <v>-24993.35664242308</v>
       </c>
       <c r="F78">
         <v>0</v>
@@ -9538,13 +9538,13 @@
         <v>2050</v>
       </c>
       <c r="C79">
-        <v>-165884.5116305721</v>
+        <v>-19965.70339844417</v>
       </c>
       <c r="D79">
-        <v>-39550.12188570197</v>
+        <v>-5.170995427761227E-05</v>
       </c>
       <c r="E79">
-        <v>-126334.3897448702</v>
+        <v>-19965.70334673417</v>
       </c>
       <c r="F79">
         <v>0</v>
@@ -9578,10 +9578,10 @@
         <v>2026</v>
       </c>
       <c r="C81">
-        <v>-164945.6975903904</v>
+        <v>-125619.4075409104</v>
       </c>
       <c r="D81">
-        <v>-39326.29020092187</v>
+        <v>-0.00015144185454119</v>
       </c>
       <c r="E81">
         <v>-125619.4073894685</v>
@@ -9598,13 +9598,13 @@
         <v>2027</v>
       </c>
       <c r="C82">
-        <v>-351912.2577443288</v>
+        <v>-232479.8352018445</v>
       </c>
       <c r="D82">
-        <v>-83902.78604103073</v>
+        <v>0.0007399740861728787</v>
       </c>
       <c r="E82">
-        <v>-268009.471703298</v>
+        <v>-232479.8359418185</v>
       </c>
       <c r="F82">
         <v>0</v>
@@ -9618,13 +9618,13 @@
         <v>2028</v>
       </c>
       <c r="C83">
-        <v>-493006.4941101348</v>
+        <v>-277768.5119118453</v>
       </c>
       <c r="D83">
-        <v>-117542.4199693934</v>
+        <v>0.001490107388235629</v>
       </c>
       <c r="E83">
-        <v>-375464.0741407414</v>
+        <v>-277768.5134019526</v>
       </c>
       <c r="F83">
         <v>0</v>
@@ -9638,13 +9638,13 @@
         <v>2029</v>
       </c>
       <c r="C84">
-        <v>-637309.606994624</v>
+        <v>-318845.7971881882</v>
       </c>
       <c r="D84">
-        <v>-151947.1130113684</v>
+        <v>0.001585987498401664</v>
       </c>
       <c r="E84">
-        <v>-485362.4939832556</v>
+        <v>-318845.7987741756</v>
       </c>
       <c r="F84">
         <v>0</v>
@@ -9658,13 +9658,13 @@
         <v>2030</v>
       </c>
       <c r="C85">
-        <v>-824566.607211889</v>
+        <v>-387632.4814376342</v>
       </c>
       <c r="D85">
-        <v>-196592.8554604111</v>
+        <v>0.001726074740872718</v>
       </c>
       <c r="E85">
-        <v>-627973.7517514778</v>
+        <v>-387632.4831637088</v>
       </c>
       <c r="F85">
         <v>0</v>
@@ -9678,13 +9678,13 @@
         <v>2031</v>
       </c>
       <c r="C86">
-        <v>-995392.2324644178</v>
+        <v>-431342.7384104711</v>
       </c>
       <c r="D86">
-        <v>-237321.0357680753</v>
+        <v>0.001261452154722065</v>
       </c>
       <c r="E86">
-        <v>-758071.1966963424</v>
+        <v>-431342.739671923</v>
       </c>
       <c r="F86">
         <v>0</v>
@@ -9698,13 +9698,13 @@
         <v>2032</v>
       </c>
       <c r="C87">
-        <v>-1197429.252003672</v>
+        <v>-494384.6446957145</v>
       </c>
       <c r="D87">
-        <v>-285490.624777064</v>
+        <v>0.001417817053152248</v>
       </c>
       <c r="E87">
-        <v>-911938.6272266083</v>
+        <v>-494384.6461135314</v>
       </c>
       <c r="F87">
         <v>0</v>
@@ -9718,13 +9718,13 @@
         <v>2033</v>
       </c>
       <c r="C88">
-        <v>-1386991.56151479</v>
+        <v>-538196.018986236</v>
       </c>
       <c r="D88">
-        <v>-330685.9981871886</v>
+        <v>0.001494403069955297</v>
       </c>
       <c r="E88">
-        <v>-1056305.563327602</v>
+        <v>-538196.0204806388</v>
       </c>
       <c r="F88">
         <v>0</v>
@@ -9738,13 +9738,13 @@
         <v>2034</v>
       </c>
       <c r="C89">
-        <v>-1595182.695949129</v>
+        <v>-592608.0496019826</v>
       </c>
       <c r="D89">
-        <v>-380322.8489182437</v>
+        <v>0.0009028703061630949</v>
       </c>
       <c r="E89">
-        <v>-1214859.847030886</v>
+        <v>-592608.0505048528</v>
       </c>
       <c r="F89">
         <v>0</v>
@@ -9758,13 +9758,13 @@
         <v>2035</v>
       </c>
       <c r="C90">
-        <v>-1776735.474180181</v>
+        <v>-620207.6430454489</v>
       </c>
       <c r="D90">
-        <v>-423608.5929406685</v>
+        <v>0.0008298105967696756</v>
       </c>
       <c r="E90">
-        <v>-1353126.881239512</v>
+        <v>-620207.6438752594</v>
       </c>
       <c r="F90">
         <v>0</v>
@@ -9778,13 +9778,13 @@
         <v>2036</v>
       </c>
       <c r="C91">
-        <v>-1947551.234270046</v>
+        <v>-641042.8694042794</v>
       </c>
       <c r="D91">
-        <v>-464334.4212000196</v>
+        <v>0.000449105937150307</v>
       </c>
       <c r="E91">
-        <v>-1483216.813070026</v>
+        <v>-641042.8698533853</v>
       </c>
       <c r="F91">
         <v>0</v>
@@ -9798,13 +9798,13 @@
         <v>2037</v>
       </c>
       <c r="C92">
-        <v>-2116427.999477262</v>
+        <v>-663268.0327813387</v>
       </c>
       <c r="D92">
-        <v>-504597.955040255</v>
+        <v>0.0004372939583845437</v>
       </c>
       <c r="E92">
-        <v>-1611830.044437007</v>
+        <v>-663268.0332186325</v>
       </c>
       <c r="F92">
         <v>0</v>
@@ -9818,13 +9818,13 @@
         <v>2038</v>
       </c>
       <c r="C93">
-        <v>-2315860.333421328</v>
+        <v>-710646.8979519003</v>
       </c>
       <c r="D93">
-        <v>-552146.535904776</v>
+        <v>-0.0002585464244475588</v>
       </c>
       <c r="E93">
-        <v>-1763713.797516552</v>
+        <v>-710646.8976933537</v>
       </c>
       <c r="F93">
         <v>0</v>
@@ -9838,13 +9838,13 @@
         <v>2039</v>
       </c>
       <c r="C94">
-        <v>-2506712.911195666</v>
+        <v>-745789.6550354722</v>
       </c>
       <c r="D94">
-        <v>-597649.5345812622</v>
+        <v>-2.861687971744686E-05</v>
       </c>
       <c r="E94">
-        <v>-1909063.376614404</v>
+        <v>-745789.655006855</v>
       </c>
       <c r="F94">
         <v>0</v>
@@ -9858,13 +9858,13 @@
         <v>2040</v>
       </c>
       <c r="C95">
-        <v>-2672036.647915808</v>
+        <v>-759560.3519824781</v>
       </c>
       <c r="D95">
-        <v>-637065.9567270672</v>
+        <v>-0.0001188020978588611</v>
       </c>
       <c r="E95">
-        <v>-2034970.691188741</v>
+        <v>-759560.3518636755</v>
       </c>
       <c r="F95">
         <v>0</v>
@@ -9878,13 +9878,13 @@
         <v>2041</v>
       </c>
       <c r="C96">
-        <v>-2877006.309176486</v>
+        <v>-807559.3332018215</v>
       </c>
       <c r="D96">
-        <v>-685934.7450548427</v>
+        <v>-0.0001590863103047013</v>
       </c>
       <c r="E96">
-        <v>-2191071.564121643</v>
+        <v>-807559.3330427348</v>
       </c>
       <c r="F96">
         <v>0</v>
@@ -9898,13 +9898,13 @@
         <v>2042</v>
       </c>
       <c r="C97">
-        <v>-3044132.068494089</v>
+        <v>-820411.1164683136</v>
       </c>
       <c r="D97">
-        <v>-725780.8047398599</v>
+        <v>0.0001141807006206363</v>
       </c>
       <c r="E97">
-        <v>-2318351.263754229</v>
+        <v>-820411.1165824938</v>
       </c>
       <c r="F97">
         <v>0</v>
@@ -9918,13 +9918,13 @@
         <v>2043</v>
       </c>
       <c r="C98">
-        <v>-3226755.449528381</v>
+        <v>-849070.1988448948</v>
       </c>
       <c r="D98">
-        <v>-769321.8014736024</v>
+        <v>0.0006978782039368525</v>
       </c>
       <c r="E98">
-        <v>-2457433.648054778</v>
+        <v>-849070.1995427725</v>
       </c>
       <c r="F98">
         <v>0</v>
@@ -9938,13 +9938,13 @@
         <v>2044</v>
       </c>
       <c r="C99">
-        <v>-3402750.753861025</v>
+        <v>-871548.4436049144</v>
       </c>
       <c r="D99">
-        <v>-811282.5346924381</v>
+        <v>0.001380694724502973</v>
       </c>
       <c r="E99">
-        <v>-2591468.219168586</v>
+        <v>-871548.4449856086</v>
       </c>
       <c r="F99">
         <v>0</v>
@@ -9958,13 +9958,13 @@
         <v>2045</v>
       </c>
       <c r="C100">
-        <v>-3559016.516709119</v>
+        <v>-879491.1013640384</v>
       </c>
       <c r="D100">
-        <v>-848539.3581683274</v>
+        <v>0.001735345635097474</v>
       </c>
       <c r="E100">
-        <v>-2710477.15854079</v>
+        <v>-879491.1030993834</v>
       </c>
       <c r="F100">
         <v>0</v>
@@ -9978,13 +9978,13 @@
         <v>2046</v>
       </c>
       <c r="C101">
-        <v>-3719135.96477867</v>
+        <v>-894685.1893030966</v>
       </c>
       <c r="D101">
-        <v>-886714.9758023908</v>
+        <v>0.002504240575945005</v>
       </c>
       <c r="E101">
-        <v>-2832420.988976278</v>
+        <v>-894685.1918073365</v>
       </c>
       <c r="F101">
         <v>0</v>
@@ -9998,13 +9998,13 @@
         <v>2047</v>
       </c>
       <c r="C102">
-        <v>-3894013.51439266</v>
+        <v>-922723.043066513</v>
       </c>
       <c r="D102">
-        <v>-928409.2143682506</v>
+        <v>0.002663787250639871</v>
       </c>
       <c r="E102">
-        <v>-2965604.300024409</v>
+        <v>-922723.0457302995</v>
       </c>
       <c r="F102">
         <v>0</v>
@@ -10018,13 +10018,13 @@
         <v>2048</v>
       </c>
       <c r="C103">
-        <v>-4071270.987135202</v>
+        <v>-950180.3057621896</v>
       </c>
       <c r="D103">
-        <v>-970670.8732971546</v>
+        <v>0.002801838199957274</v>
       </c>
       <c r="E103">
-        <v>-3100600.113838047</v>
+        <v>-950180.3085640271</v>
       </c>
       <c r="F103">
         <v>0</v>
@@ -10038,13 +10038,13 @@
         <v>2049</v>
       </c>
       <c r="C104">
-        <v>-4215625.997774689</v>
+        <v>-950402.2769517931</v>
       </c>
       <c r="D104">
-        <v>-1005087.939782048</v>
+        <v>0.003530991176376119</v>
       </c>
       <c r="E104">
-        <v>-3210538.057992641</v>
+        <v>-950402.2804827837</v>
       </c>
       <c r="F104">
         <v>0</v>
@@ -10058,13 +10058,13 @@
         <v>2050</v>
       </c>
       <c r="C105">
-        <v>-4385215.090940268</v>
+        <v>-975395.6337047939</v>
       </c>
       <c r="D105">
-        <v>-1045521.306581967</v>
+        <v>0.003420413442654535</v>
       </c>
       <c r="E105">
-        <v>-3339693.7843583</v>
+        <v>-975395.6371252068</v>
       </c>
       <c r="F105">
         <v>0</v>
@@ -10078,10 +10078,10 @@
         <v>2025</v>
       </c>
       <c r="C106">
-        <v>280902.071782</v>
+        <v>241575.78173252</v>
       </c>
       <c r="D106">
-        <v>39326.29004948001</v>
+        <v>0</v>
       </c>
       <c r="E106">
         <v>241575.78173252</v>
@@ -10098,16 +10098,16 @@
         <v>2026</v>
       </c>
       <c r="C107">
-        <v>318403.54808232</v>
+        <v>205500.8287325655</v>
       </c>
       <c r="D107">
-        <v>44576.49673152481</v>
+        <v>0</v>
       </c>
       <c r="E107">
-        <v>273827.0513507952</v>
+        <v>205500.8287325655</v>
       </c>
       <c r="F107">
-        <v>131436.9846483817</v>
+        <v>98640.39779163145</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -10118,16 +10118,16 @@
         <v>2027</v>
       </c>
       <c r="C108">
-        <v>240283.1048464</v>
+        <v>87093.61444230931</v>
       </c>
       <c r="D108">
-        <v>33639.634678496</v>
+        <v>0</v>
       </c>
       <c r="E108">
-        <v>206643.470167904</v>
+        <v>87093.61444230932</v>
       </c>
       <c r="F108">
-        <v>99188.86568059392</v>
+        <v>41804.93493230848</v>
       </c>
     </row>
     <row r="109" spans="1:6">
@@ -10138,16 +10138,16 @@
         <v>2028</v>
       </c>
       <c r="C109">
-        <v>245747.808127536</v>
+        <v>78994.77946989023</v>
       </c>
       <c r="D109">
-        <v>34404.69313785505</v>
+        <v>0</v>
       </c>
       <c r="E109">
-        <v>211343.114989681</v>
+        <v>78994.77946989026</v>
       </c>
       <c r="F109">
-        <v>101444.6951950469</v>
+        <v>37917.49414554733</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -10158,16 +10158,16 @@
         <v>2029</v>
       </c>
       <c r="C110">
-        <v>318898.161350928</v>
+        <v>132282.0853412421</v>
       </c>
       <c r="D110">
-        <v>44645.74258912993</v>
+        <v>0</v>
       </c>
       <c r="E110">
-        <v>274252.4187617981</v>
+        <v>132282.0853412421</v>
       </c>
       <c r="F110">
-        <v>131641.1610056631</v>
+        <v>63495.40096379622</v>
       </c>
     </row>
     <row r="111" spans="1:6">
@@ -10178,16 +10178,16 @@
         <v>2030</v>
       </c>
       <c r="C111">
-        <v>290915.57030744</v>
+        <v>84058.18193237856</v>
       </c>
       <c r="D111">
-        <v>40728.1798430416</v>
+        <v>0</v>
       </c>
       <c r="E111">
-        <v>250187.3904643984</v>
+        <v>84058.18193237856</v>
       </c>
       <c r="F111">
-        <v>120089.9474229112</v>
+        <v>40347.92732754172</v>
       </c>
     </row>
     <row r="112" spans="1:6">
@@ -10198,16 +10198,16 @@
         <v>2031</v>
       </c>
       <c r="C112">
-        <v>344068.4940382401</v>
+        <v>121234.4354716221</v>
       </c>
       <c r="D112">
-        <v>48169.58916535361</v>
+        <v>0</v>
       </c>
       <c r="E112">
-        <v>295898.9048728864</v>
+        <v>121234.4354716221</v>
       </c>
       <c r="F112">
-        <v>142031.4743389855</v>
+        <v>58192.5290263786</v>
       </c>
     </row>
     <row r="113" spans="1:6">
@@ -10218,16 +10218,16 @@
         <v>2032</v>
       </c>
       <c r="C113">
-        <v>322824.096333648</v>
+        <v>84252.64258946435</v>
       </c>
       <c r="D113">
-        <v>45195.37348671073</v>
+        <v>0</v>
       </c>
       <c r="E113">
-        <v>277628.7228469373</v>
+        <v>84252.64258946438</v>
       </c>
       <c r="F113">
-        <v>133261.7869665299</v>
+        <v>40441.26844294291</v>
       </c>
     </row>
     <row r="114" spans="1:6">
@@ -10238,16 +10238,16 @@
         <v>2033</v>
       </c>
       <c r="C114">
-        <v>354548.929568016</v>
+        <v>104638.5146610513</v>
       </c>
       <c r="D114">
-        <v>49636.85013952225</v>
+        <v>0</v>
       </c>
       <c r="E114">
-        <v>304912.0794284938</v>
+        <v>104638.5146610513</v>
       </c>
       <c r="F114">
-        <v>146357.798125677</v>
+        <v>50226.4870373046</v>
       </c>
     </row>
     <row r="115" spans="1:6">
@@ -10258,16 +10258,16 @@
         <v>2034</v>
       </c>
       <c r="C115">
-        <v>309183.885352608</v>
+        <v>53076.13979128154</v>
       </c>
       <c r="D115">
-        <v>43285.74394936513</v>
+        <v>0</v>
       </c>
       <c r="E115">
-        <v>265898.1414032429</v>
+        <v>53076.13979128154</v>
       </c>
       <c r="F115">
-        <v>127631.1078735566</v>
+        <v>25476.54709981513</v>
       </c>
     </row>
     <row r="116" spans="1:6">
@@ -10278,16 +10278,16 @@
         <v>2035</v>
       </c>
       <c r="C116">
-        <v>290898.77056176</v>
+        <v>40067.7391208277</v>
       </c>
       <c r="D116">
-        <v>40725.82787864641</v>
+        <v>0</v>
       </c>
       <c r="E116">
-        <v>250172.9426831136</v>
+        <v>40067.7391208277</v>
       </c>
       <c r="F116">
-        <v>120083.0124878945</v>
+        <v>19232.5147779973</v>
       </c>
     </row>
     <row r="117" spans="1:6">
@@ -10298,16 +10298,16 @@
         <v>2036</v>
       </c>
       <c r="C117">
-        <v>287596.670203024</v>
+        <v>42740.69790972929</v>
       </c>
       <c r="D117">
-        <v>40263.53382842337</v>
+        <v>0</v>
       </c>
       <c r="E117">
-        <v>247333.1363746006</v>
+        <v>42740.69790972929</v>
       </c>
       <c r="F117">
-        <v>118719.9054598083</v>
+        <v>20515.53499667006</v>
       </c>
     </row>
     <row r="118" spans="1:6">
@@ -10318,16 +10318,16 @@
         <v>2037</v>
       </c>
       <c r="C118">
-        <v>339632.715490576</v>
+        <v>91113.1956972339</v>
       </c>
       <c r="D118">
-        <v>47548.58016868064</v>
+        <v>0</v>
       </c>
       <c r="E118">
-        <v>292084.1353218954</v>
+        <v>91113.19569723392</v>
       </c>
       <c r="F118">
-        <v>140200.3849545098</v>
+        <v>43734.33393467228</v>
       </c>
     </row>
     <row r="119" spans="1:6">
@@ -10338,16 +10338,16 @@
         <v>2038</v>
       </c>
       <c r="C119">
-        <v>325021.420760112</v>
+        <v>67582.22611456132</v>
       </c>
       <c r="D119">
-        <v>45502.99890641568</v>
+        <v>0</v>
       </c>
       <c r="E119">
-        <v>279518.4218536963</v>
+        <v>67582.22611456129</v>
       </c>
       <c r="F119">
-        <v>134168.8424897742</v>
+        <v>32439.46853498943</v>
       </c>
     </row>
     <row r="120" spans="1:6">
@@ -10358,16 +10358,16 @@
         <v>2039</v>
       </c>
       <c r="C120">
-        <v>281545.871825856</v>
+        <v>26482.10800578038</v>
       </c>
       <c r="D120">
-        <v>39416.42205561985</v>
+        <v>0</v>
       </c>
       <c r="E120">
-        <v>242129.4497702362</v>
+        <v>26482.10800578038</v>
       </c>
       <c r="F120">
-        <v>116222.1358897134</v>
+        <v>12711.4118427746</v>
       </c>
     </row>
     <row r="121" spans="1:6">
@@ -10378,16 +10378,16 @@
         <v>2040</v>
       </c>
       <c r="C121">
-        <v>349062.77348208</v>
+        <v>92305.73182181444</v>
       </c>
       <c r="D121">
-        <v>48868.78828749121</v>
+        <v>0</v>
       </c>
       <c r="E121">
-        <v>300193.9851945888</v>
+        <v>92305.73182181446</v>
       </c>
       <c r="F121">
-        <v>144093.1128934026</v>
+        <v>44306.75127447094</v>
       </c>
     </row>
     <row r="122" spans="1:6">
@@ -10398,16 +10398,16 @@
         <v>2041</v>
       </c>
       <c r="C122">
-        <v>284614.713987744</v>
+        <v>24714.9692355615</v>
       </c>
       <c r="D122">
-        <v>39846.05995828417</v>
+        <v>0</v>
       </c>
       <c r="E122">
-        <v>244768.6540294598</v>
+        <v>24714.9692355615</v>
       </c>
       <c r="F122">
-        <v>117488.9539341407</v>
+        <v>11863.18523306953</v>
       </c>
     </row>
     <row r="123" spans="1:6">
@@ -10418,16 +10418,16 @@
         <v>2042</v>
       </c>
       <c r="C123">
-        <v>311007.123696</v>
+        <v>55113.62380111747</v>
       </c>
       <c r="D123">
-        <v>43540.99731744001</v>
+        <v>0</v>
       </c>
       <c r="E123">
-        <v>267466.12637856</v>
+        <v>55113.62380111747</v>
       </c>
       <c r="F123">
-        <v>128383.7406617088</v>
+        <v>26454.53942453639</v>
       </c>
     </row>
     <row r="124" spans="1:6">
@@ -10438,16 +10438,16 @@
         <v>2043</v>
       </c>
       <c r="C124">
-        <v>299719.527868944</v>
+        <v>43227.3984461916</v>
       </c>
       <c r="D124">
-        <v>41960.73390165217</v>
+        <v>0</v>
       </c>
       <c r="E124">
-        <v>257758.7939672919</v>
+        <v>43227.39844619163</v>
       </c>
       <c r="F124">
-        <v>123724.2211043001</v>
+        <v>20749.15125417199</v>
       </c>
     </row>
     <row r="125" spans="1:6">
@@ -10458,16 +10458,16 @@
         <v>2044</v>
       </c>
       <c r="C125">
-        <v>266120.170218144</v>
+        <v>15274.34396754619</v>
       </c>
       <c r="D125">
-        <v>37256.82383054017</v>
+        <v>0</v>
       </c>
       <c r="E125">
-        <v>228863.3463876038</v>
+        <v>15274.34396754616</v>
       </c>
       <c r="F125">
-        <v>109854.4062660498</v>
+        <v>7331.685104422155</v>
       </c>
     </row>
     <row r="126" spans="1:6">
@@ -10478,16 +10478,16 @@
         <v>2045</v>
       </c>
       <c r="C126">
-        <v>272682.9885925601</v>
+        <v>29219.40532895818</v>
       </c>
       <c r="D126">
-        <v>38175.61840295841</v>
+        <v>0</v>
       </c>
       <c r="E126">
-        <v>234507.3701896016</v>
+        <v>29219.40532895818</v>
       </c>
       <c r="F126">
-        <v>112563.5376910088</v>
+        <v>14025.31455789994</v>
       </c>
     </row>
     <row r="127" spans="1:6">
@@ -10498,16 +10498,16 @@
         <v>2046</v>
       </c>
       <c r="C127">
-        <v>297815.99089576</v>
+        <v>53918.95000656991</v>
       </c>
       <c r="D127">
-        <v>41694.23872540641</v>
+        <v>0</v>
       </c>
       <c r="E127">
-        <v>256121.7521703536</v>
+        <v>53918.95000656991</v>
       </c>
       <c r="F127">
-        <v>122938.4410417697</v>
+        <v>25881.09600315357</v>
       </c>
     </row>
     <row r="128" spans="1:6">
@@ -10518,16 +10518,16 @@
         <v>2047</v>
       </c>
       <c r="C128">
-        <v>301868.993335392</v>
+        <v>52802.42853783947</v>
       </c>
       <c r="D128">
-        <v>42261.65906695489</v>
+        <v>0</v>
       </c>
       <c r="E128">
-        <v>259607.3342684371</v>
+        <v>52802.42853783947</v>
       </c>
       <c r="F128">
-        <v>124611.5204488498</v>
+        <v>25345.16569816295</v>
       </c>
     </row>
     <row r="129" spans="1:6">
@@ -10538,16 +10538,16 @@
         <v>2048</v>
       </c>
       <c r="C129">
-        <v>245836.194386048</v>
+        <v>426.8728723146196</v>
       </c>
       <c r="D129">
-        <v>34417.06721404673</v>
+        <v>0</v>
       </c>
       <c r="E129">
-        <v>211419.1271720013</v>
+        <v>426.8728723146196</v>
       </c>
       <c r="F129">
-        <v>101481.1810425606</v>
+        <v>204.8989787110186</v>
       </c>
     </row>
     <row r="130" spans="1:6">
@@ -10558,16 +10558,16 @@
         <v>2049</v>
       </c>
       <c r="C130">
-        <v>288809.76206672</v>
+        <v>48064.14590961693</v>
       </c>
       <c r="D130">
-        <v>40433.3666893408</v>
+        <v>0</v>
       </c>
       <c r="E130">
-        <v>248376.3953773792</v>
+        <v>48064.14590961693</v>
       </c>
       <c r="F130">
-        <v>119220.669781142</v>
+        <v>23070.79003661613</v>
       </c>
     </row>
     <row r="131" spans="1:6">
@@ -10578,16 +10578,16 @@
         <v>2050</v>
       </c>
       <c r="C131">
-        <v>282500.8702428</v>
+        <v>38395.58225854655</v>
       </c>
       <c r="D131">
-        <v>39550.12183399201</v>
+        <v>0</v>
       </c>
       <c r="E131">
-        <v>242950.748408808</v>
+        <v>38395.58225854652</v>
       </c>
       <c r="F131">
-        <v>116616.3592362279</v>
+        <v>18429.87948410233</v>
       </c>
     </row>
     <row r="132" spans="1:6">
@@ -10618,10 +10618,10 @@
         <v>2026</v>
       </c>
       <c r="C133">
-        <v>280902.071782</v>
+        <v>241575.78173252</v>
       </c>
       <c r="D133">
-        <v>39326.29004948001</v>
+        <v>0</v>
       </c>
       <c r="E133">
         <v>241575.78173252</v>
@@ -10638,16 +10638,16 @@
         <v>2027</v>
       </c>
       <c r="C134">
-        <v>599305.61986432</v>
+        <v>447076.6104650855</v>
       </c>
       <c r="D134">
-        <v>83902.7867810048</v>
+        <v>0</v>
       </c>
       <c r="E134">
-        <v>515402.8330833152</v>
+        <v>447076.6104650855</v>
       </c>
       <c r="F134">
-        <v>247393.3598799913</v>
+        <v>214596.7730232411</v>
       </c>
     </row>
     <row r="135" spans="1:6">
@@ -10658,16 +10658,16 @@
         <v>2028</v>
       </c>
       <c r="C135">
-        <v>839588.72471072</v>
+        <v>534170.2249073947</v>
       </c>
       <c r="D135">
-        <v>117542.4214595008</v>
+        <v>0</v>
       </c>
       <c r="E135">
-        <v>722046.3032512192</v>
+        <v>534170.2249073948</v>
       </c>
       <c r="F135">
-        <v>346582.2255605853</v>
+        <v>256401.7079555495</v>
       </c>
     </row>
     <row r="136" spans="1:6">
@@ -10678,16 +10678,16 @@
         <v>2029</v>
       </c>
       <c r="C136">
-        <v>1085336.532838256</v>
+        <v>613165.004377285</v>
       </c>
       <c r="D136">
-        <v>151947.1145973559</v>
+        <v>0</v>
       </c>
       <c r="E136">
-        <v>933389.4182409002</v>
+        <v>613165.0043772851</v>
       </c>
       <c r="F136">
-        <v>448026.9207556322</v>
+        <v>294319.2021010969</v>
       </c>
     </row>
     <row r="137" spans="1:6">
@@ -10698,16 +10698,16 @@
         <v>2030</v>
       </c>
       <c r="C137">
-        <v>1404234.694189184</v>
+        <v>745447.0897185272</v>
       </c>
       <c r="D137">
-        <v>196592.8571864858</v>
+        <v>0</v>
       </c>
       <c r="E137">
-        <v>1207641.837002698</v>
+        <v>745447.0897185273</v>
       </c>
       <c r="F137">
-        <v>579668.0817612952</v>
+        <v>357814.603064893</v>
       </c>
     </row>
     <row r="138" spans="1:6">
@@ -10718,16 +10718,16 @@
         <v>2031</v>
       </c>
       <c r="C138">
-        <v>1695150.264496624</v>
+        <v>829505.2716509057</v>
       </c>
       <c r="D138">
-        <v>237321.0370295274</v>
+        <v>0</v>
       </c>
       <c r="E138">
-        <v>1457829.227467097</v>
+        <v>829505.2716509058</v>
       </c>
       <c r="F138">
-        <v>699758.0291842064</v>
+        <v>398162.5303924348</v>
       </c>
     </row>
     <row r="139" spans="1:6">
@@ -10738,16 +10738,16 @@
         <v>2032</v>
       </c>
       <c r="C139">
-        <v>2039218.758534864</v>
+        <v>950739.7071225278</v>
       </c>
       <c r="D139">
-        <v>285490.626194881</v>
+        <v>0</v>
       </c>
       <c r="E139">
-        <v>1753728.132339983</v>
+        <v>950739.7071225279</v>
       </c>
       <c r="F139">
-        <v>841789.5035231919</v>
+        <v>456355.0594188134</v>
       </c>
     </row>
     <row r="140" spans="1:6">
@@ -10758,16 +10758,16 @@
         <v>2033</v>
       </c>
       <c r="C140">
-        <v>2362042.854868512</v>
+        <v>1034992.349711992</v>
       </c>
       <c r="D140">
-        <v>330685.9996815917</v>
+        <v>0</v>
       </c>
       <c r="E140">
-        <v>2031356.85518692</v>
+        <v>1034992.349711992</v>
       </c>
       <c r="F140">
-        <v>975051.2904897218</v>
+        <v>496796.3278617563</v>
       </c>
     </row>
     <row r="141" spans="1:6">
@@ -10778,16 +10778,16 @@
         <v>2034</v>
       </c>
       <c r="C141">
-        <v>2716591.784436528</v>
+        <v>1139630.864373043</v>
       </c>
       <c r="D141">
-        <v>380322.8498211139</v>
+        <v>0</v>
       </c>
       <c r="E141">
-        <v>2336268.934615414</v>
+        <v>1139630.864373044</v>
       </c>
       <c r="F141">
-        <v>1121409.088615399</v>
+        <v>547022.8148990609</v>
       </c>
     </row>
     <row r="142" spans="1:6">
@@ -10798,16 +10798,16 @@
         <v>2035</v>
       </c>
       <c r="C142">
-        <v>3025775.669789136</v>
+        <v>1192707.004164325</v>
       </c>
       <c r="D142">
-        <v>423608.5937704791</v>
+        <v>0</v>
       </c>
       <c r="E142">
-        <v>2602167.076018657</v>
+        <v>1192707.004164325</v>
       </c>
       <c r="F142">
-        <v>1249040.196488956</v>
+        <v>572499.361998876</v>
       </c>
     </row>
     <row r="143" spans="1:6">
@@ -10818,16 +10818,16 @@
         <v>2036</v>
       </c>
       <c r="C143">
-        <v>3316674.440350896</v>
+        <v>1232774.743285153</v>
       </c>
       <c r="D143">
-        <v>464334.4216491255</v>
+        <v>0</v>
       </c>
       <c r="E143">
-        <v>2852340.018701771</v>
+        <v>1232774.743285153</v>
       </c>
       <c r="F143">
-        <v>1369123.20897685</v>
+        <v>591731.8767768733</v>
       </c>
     </row>
     <row r="144" spans="1:6">
@@ -10838,16 +10838,16 @@
         <v>2037</v>
       </c>
       <c r="C144">
-        <v>3604271.11055392</v>
+        <v>1275515.441194882</v>
       </c>
       <c r="D144">
-        <v>504597.9554775489</v>
+        <v>0</v>
       </c>
       <c r="E144">
-        <v>3099673.155076372</v>
+        <v>1275515.441194882</v>
       </c>
       <c r="F144">
-        <v>1487843.114436659</v>
+        <v>612247.4117735433</v>
       </c>
     </row>
     <row r="145" spans="1:6">
@@ -10858,16 +10858,16 @@
         <v>2038</v>
       </c>
       <c r="C145">
-        <v>3943903.826044496</v>
+        <v>1366628.636892116</v>
       </c>
       <c r="D145">
-        <v>552146.5356462295</v>
+        <v>0</v>
       </c>
       <c r="E145">
-        <v>3391757.290398267</v>
+        <v>1366628.636892116</v>
       </c>
       <c r="F145">
-        <v>1628043.499391168</v>
+        <v>655981.7457082156</v>
       </c>
     </row>
     <row r="146" spans="1:6">
@@ -10878,16 +10878,16 @@
         <v>2039</v>
       </c>
       <c r="C146">
-        <v>4268925.246804608</v>
+        <v>1434210.863006677</v>
       </c>
       <c r="D146">
-        <v>597649.5345526452</v>
+        <v>0</v>
       </c>
       <c r="E146">
-        <v>3671275.712251964</v>
+        <v>1434210.863006677</v>
       </c>
       <c r="F146">
-        <v>1762212.341880943</v>
+        <v>688421.214243205</v>
       </c>
     </row>
     <row r="147" spans="1:6">
@@ -10898,16 +10898,16 @@
         <v>2040</v>
       </c>
       <c r="C147">
-        <v>4550471.118630464</v>
+        <v>1460692.971012458</v>
       </c>
       <c r="D147">
-        <v>637065.9566082651</v>
+        <v>0</v>
       </c>
       <c r="E147">
-        <v>3913405.1620222</v>
+        <v>1460692.971012458</v>
       </c>
       <c r="F147">
-        <v>1878434.477770656</v>
+        <v>701132.6260859796</v>
       </c>
     </row>
     <row r="148" spans="1:6">
@@ -10918,16 +10918,16 @@
         <v>2041</v>
       </c>
       <c r="C148">
-        <v>4899533.892112544</v>
+        <v>1552998.702834272</v>
       </c>
       <c r="D148">
-        <v>685934.7448957562</v>
+        <v>0</v>
       </c>
       <c r="E148">
-        <v>4213599.147216788</v>
+        <v>1552998.702834272</v>
       </c>
       <c r="F148">
-        <v>2022527.590664059</v>
+        <v>745439.3773604506</v>
       </c>
     </row>
     <row r="149" spans="1:6">
@@ -10938,16 +10938,16 @@
         <v>2042</v>
       </c>
       <c r="C149">
-        <v>5184148.606100288</v>
+        <v>1577713.672069834</v>
       </c>
       <c r="D149">
-        <v>725780.8048540404</v>
+        <v>0</v>
       </c>
       <c r="E149">
-        <v>4458367.801246248</v>
+        <v>1577713.672069834</v>
       </c>
       <c r="F149">
-        <v>2140016.544598199</v>
+        <v>757302.5625935202</v>
       </c>
     </row>
     <row r="150" spans="1:6">
@@ -10958,16 +10958,16 @@
         <v>2043</v>
       </c>
       <c r="C150">
-        <v>5495155.729796289</v>
+        <v>1632827.295870951</v>
       </c>
       <c r="D150">
-        <v>769321.8021714804</v>
+        <v>0</v>
       </c>
       <c r="E150">
-        <v>4725833.927624809</v>
+        <v>1632827.295870951</v>
       </c>
       <c r="F150">
-        <v>2268400.285259908</v>
+        <v>783757.1020180566</v>
       </c>
     </row>
     <row r="151" spans="1:6">
@@ -10978,16 +10978,16 @@
         <v>2044</v>
       </c>
       <c r="C151">
-        <v>5794875.257665233</v>
+        <v>1676054.694317143</v>
       </c>
       <c r="D151">
-        <v>811282.5360731325</v>
+        <v>0</v>
       </c>
       <c r="E151">
-        <v>4983592.7215921</v>
+        <v>1676054.694317143</v>
       </c>
       <c r="F151">
-        <v>2392124.506364208</v>
+        <v>804506.2532722285</v>
       </c>
     </row>
     <row r="152" spans="1:6">
@@ -10998,16 +10998,16 @@
         <v>2045</v>
       </c>
       <c r="C152">
-        <v>6060995.427883376</v>
+        <v>1691329.038284689</v>
       </c>
       <c r="D152">
-        <v>848539.3599036727</v>
+        <v>0</v>
       </c>
       <c r="E152">
-        <v>5212456.067979705</v>
+        <v>1691329.038284689</v>
       </c>
       <c r="F152">
-        <v>2501978.912630258</v>
+        <v>811837.9383766507</v>
       </c>
     </row>
     <row r="153" spans="1:6">
@@ -11018,16 +11018,16 @@
         <v>2046</v>
       </c>
       <c r="C153">
-        <v>6333678.416475937</v>
+        <v>1720548.443613647</v>
       </c>
       <c r="D153">
-        <v>886714.9783066311</v>
+        <v>0</v>
       </c>
       <c r="E153">
-        <v>5446963.438169306</v>
+        <v>1720548.443613647</v>
       </c>
       <c r="F153">
-        <v>2614542.450321267</v>
+        <v>825863.2529345506</v>
       </c>
     </row>
     <row r="154" spans="1:6">
@@ -11038,16 +11038,16 @@
         <v>2047</v>
       </c>
       <c r="C154">
-        <v>6631494.407371697</v>
+        <v>1774467.393620217</v>
       </c>
       <c r="D154">
-        <v>928409.2170320374</v>
+        <v>0</v>
       </c>
       <c r="E154">
-        <v>5703085.190339659</v>
+        <v>1774467.393620217</v>
       </c>
       <c r="F154">
-        <v>2737480.891363037</v>
+        <v>851744.3489377042</v>
       </c>
     </row>
     <row r="155" spans="1:6">
@@ -11058,16 +11058,16 @@
         <v>2048</v>
       </c>
       <c r="C155">
-        <v>6933363.400707089</v>
+        <v>1827269.822158057</v>
       </c>
       <c r="D155">
-        <v>970670.8760989923</v>
+        <v>0</v>
       </c>
       <c r="E155">
-        <v>5962692.524608096</v>
+        <v>1827269.822158057</v>
       </c>
       <c r="F155">
-        <v>2862092.411811887</v>
+        <v>877089.5146358672</v>
       </c>
     </row>
     <row r="156" spans="1:6">
@@ -11078,16 +11078,16 @@
         <v>2049</v>
       </c>
       <c r="C156">
-        <v>7179199.595093138</v>
+        <v>1827696.695030372</v>
       </c>
       <c r="D156">
-        <v>1005087.943313039</v>
+        <v>0</v>
       </c>
       <c r="E156">
-        <v>6174111.651780098</v>
+        <v>1827696.695030372</v>
       </c>
       <c r="F156">
-        <v>2963573.592854448</v>
+        <v>877294.4136145782</v>
       </c>
     </row>
     <row r="157" spans="1:6">
@@ -11098,16 +11098,16 @@
         <v>2050</v>
       </c>
       <c r="C157">
-        <v>7468009.357159858</v>
+        <v>1875760.840939989</v>
       </c>
       <c r="D157">
-        <v>1045521.31000238</v>
+        <v>0</v>
       </c>
       <c r="E157">
-        <v>6422488.047157477</v>
+        <v>1875760.840939989</v>
       </c>
       <c r="F157">
-        <v>3082794.26263559</v>
+        <v>900365.2036511943</v>
       </c>
     </row>
   </sheetData>
@@ -11197,7 +11197,7 @@
         <v>37</v>
       </c>
       <c r="B10">
-        <v>0.5871999999999999</v>
+        <v>0.5872000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:2">

</xml_diff>